<commit_message>
Add US History 8-2 Module 4 to dashboard
</commit_message>
<xml_diff>
--- a/exports/US History 8-2 - Course Outline.xlsx
+++ b/exports/US History 8-2 - Course Outline.xlsx
@@ -1520,17 +1520,25 @@
       </c>
       <c r="D60" s="5"/>
       <c r="E60" s="6"/>
-      <c r="F60" s="6"/>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.6.4, 8.6.5, 8.6.6, 8.9.1, 8.9.2, 8.12.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.4, RH.6, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T5 L5 Reform and Women's Rights; T5 L6 Arts and Literature</t>
+          <t xml:space="preserve">How did reform movements, women's rights activists, artists, and writers challenge Americans to imagine a different society before the Civil War?</t>
         </is>
       </c>
       <c r="H60" s="2"/>
     </row>
     <row r="61">
       <c r="A61" s="2"/>
-      <c r="B61" s="4"/>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C61" s="5"/>
       <c r="D61" s="7" t="inlineStr">
         <is>
@@ -1544,11 +1552,15 @@
     </row>
     <row r="62">
       <c r="A62" s="2"/>
-      <c r="B62" s="4"/>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C62" s="5"/>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Reform and Women's Rights</t>
         </is>
       </c>
       <c r="E62" s="6"/>
@@ -1558,11 +1570,15 @@
     </row>
     <row r="63">
       <c r="A63" s="2"/>
-      <c r="B63" s="4"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C63" s="5"/>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Arts and Literature</t>
         </is>
       </c>
       <c r="E63" s="6"/>
@@ -1572,25 +1588,37 @@
     </row>
     <row r="64">
       <c r="A64" s="2"/>
-      <c r="B64" s="4"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C64" s="5"/>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Reform, Women's Rights, and American Culture</t>
         </is>
       </c>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
-      <c r="G64" s="6"/>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H64" s="2"/>
     </row>
     <row r="65">
       <c r="A65" s="2"/>
-      <c r="B65" s="4"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C65" s="5"/>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E65" s="6"/>
@@ -1602,15 +1630,15 @@
       <c r="A66" s="2"/>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Reform, Women's Rights &amp; Culture</t>
-        </is>
-      </c>
-      <c r="D66" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C66" s="5"/>
+      <c r="D66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Changes in American Schools</t>
+        </is>
+      </c>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
@@ -1618,85 +1646,109 @@
     </row>
     <row r="67">
       <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C67" s="5"/>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: The Early Women's Rights Movement</t>
+        </is>
+      </c>
+      <c r="E67" s="6"/>
+      <c r="F67" s="6"/>
+      <c r="G67" s="6"/>
       <c r="H67" s="2"/>
     </row>
     <row r="68">
       <c r="A68" s="2"/>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 5</t>
-        </is>
-      </c>
-      <c r="C68" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
-        </is>
-      </c>
-      <c r="D68" s="16"/>
-      <c r="E68" s="16"/>
-      <c r="F68" s="16"/>
-      <c r="G68" s="17"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C68" s="5"/>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Primary Source: Declaration of Sentiments and Resolutions</t>
+        </is>
+      </c>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
+      <c r="G68" s="6"/>
       <c r="H68" s="2"/>
     </row>
     <row r="69">
       <c r="A69" s="2"/>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
-        </is>
-      </c>
-      <c r="D69" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C69" s="5"/>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Early American Music and Literature</t>
+        </is>
+      </c>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L1 Conflicts and Compromises; T6 L2 Growing Tensions</t>
-        </is>
-      </c>
+      <c r="G69" s="6"/>
       <c r="H69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="2"/>
-      <c r="B70" s="4"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C70" s="5"/>
-      <c r="D70" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
-      <c r="G70" s="6"/>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H70" s="2"/>
     </row>
     <row r="71">
       <c r="A71" s="2"/>
-      <c r="B71" s="4"/>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C71" s="5"/>
-      <c r="D71" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Pants That Made America Panic</t>
         </is>
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
-      <c r="G71" s="6"/>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H71" s="2"/>
     </row>
     <row r="72">
       <c r="A72" s="2"/>
-      <c r="B72" s="4"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C72" s="5"/>
       <c r="D72" s="7" t="inlineStr">
         <is>
@@ -1710,27 +1762,39 @@
     </row>
     <row r="73">
       <c r="A73" s="2"/>
-      <c r="B73" s="4"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C73" s="5"/>
-      <c r="D73" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Reform, Women's Rights &amp; Culture</t>
         </is>
       </c>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
-      <c r="G73" s="6"/>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H73" s="2"/>
     </row>
     <row r="74">
       <c r="A74" s="2"/>
-      <c r="B74" s="4"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C74" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Reform, Women's Rights &amp; Culture</t>
+        </is>
+      </c>
+      <c r="D74" s="5"/>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
       <c r="G74" s="6"/>
@@ -1738,70 +1802,66 @@
     </row>
     <row r="75">
       <c r="A75" s="2"/>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
-        </is>
-      </c>
-      <c r="D75" s="5"/>
-      <c r="E75" s="6"/>
-      <c r="F75" s="6"/>
-      <c r="G75" s="6"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
       <c r="H75" s="2"/>
     </row>
     <row r="76">
       <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 5</t>
+        </is>
+      </c>
+      <c r="C76" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
+        </is>
+      </c>
+      <c r="D76" s="16"/>
+      <c r="E76" s="16"/>
+      <c r="F76" s="16"/>
+      <c r="G76" s="17"/>
       <c r="H76" s="2"/>
     </row>
     <row r="77">
       <c r="A77" s="2"/>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 6</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D77" s="16"/>
-      <c r="E77" s="16"/>
-      <c r="F77" s="16"/>
-      <c r="G77" s="17"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
+        </is>
+      </c>
+      <c r="D77" s="5"/>
+      <c r="E77" s="6"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L1 Conflicts and Compromises; T6 L2 Growing Tensions</t>
+        </is>
+      </c>
       <c r="H77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2"/>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D78" s="5"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E78" s="6"/>
       <c r="F78" s="6"/>
-      <c r="G78" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L3 Division and the Outbreak of War; T6 L4 The Course of the War</t>
-        </is>
-      </c>
+      <c r="G78" s="6"/>
       <c r="H78" s="2"/>
     </row>
     <row r="79">
@@ -1810,7 +1870,7 @@
       <c r="C79" s="5"/>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E79" s="6"/>
@@ -1824,7 +1884,7 @@
       <c r="C80" s="5"/>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E80" s="6"/>
@@ -1838,7 +1898,7 @@
       <c r="C81" s="5"/>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E81" s="6"/>
@@ -1862,13 +1922,17 @@
     </row>
     <row r="83">
       <c r="A83" s="2"/>
-      <c r="B83" s="4"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
+        </is>
+      </c>
+      <c r="D83" s="5"/>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
       <c r="G83" s="6"/>
@@ -1876,70 +1940,66 @@
     </row>
     <row r="84">
       <c r="A84" s="2"/>
-      <c r="B84" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C84" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D84" s="5"/>
-      <c r="E84" s="6"/>
-      <c r="F84" s="6"/>
-      <c r="G84" s="6"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2"/>
+      <c r="F84" s="2"/>
+      <c r="G84" s="2"/>
       <c r="H84" s="2"/>
     </row>
     <row r="85">
       <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="2"/>
-      <c r="G85" s="2"/>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 6</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D85" s="16"/>
+      <c r="E85" s="16"/>
+      <c r="F85" s="16"/>
+      <c r="G85" s="17"/>
       <c r="H85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2"/>
-      <c r="B86" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 7</t>
-        </is>
-      </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D86" s="16"/>
-      <c r="E86" s="16"/>
-      <c r="F86" s="16"/>
-      <c r="G86" s="17"/>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D86" s="5"/>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L3 Division and the Outbreak of War; T6 L4 The Course of the War</t>
+        </is>
+      </c>
       <c r="H86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2"/>
-      <c r="B87" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C87" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D87" s="5"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="5"/>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E87" s="6"/>
       <c r="F87" s="6"/>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L5 Emancipation and Life in Wartime</t>
-        </is>
-      </c>
+      <c r="G87" s="6"/>
       <c r="H87" s="2"/>
     </row>
     <row r="88">
@@ -1948,7 +2008,7 @@
       <c r="C88" s="5"/>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E88" s="6"/>
@@ -1962,7 +2022,7 @@
       <c r="C89" s="5"/>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E89" s="6"/>
@@ -1976,7 +2036,7 @@
       <c r="C90" s="5"/>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E90" s="6"/>
@@ -2000,13 +2060,17 @@
     </row>
     <row r="92">
       <c r="A92" s="2"/>
-      <c r="B92" s="4"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D92" s="5"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
       <c r="G92" s="6"/>
@@ -2014,70 +2078,66 @@
     </row>
     <row r="93">
       <c r="A93" s="2"/>
-      <c r="B93" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C93" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D93" s="5"/>
-      <c r="E93" s="6"/>
-      <c r="F93" s="6"/>
-      <c r="G93" s="6"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
       <c r="H93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-      <c r="E94" s="2"/>
-      <c r="F94" s="2"/>
-      <c r="G94" s="2"/>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 7</t>
+        </is>
+      </c>
+      <c r="C94" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D94" s="16"/>
+      <c r="E94" s="16"/>
+      <c r="F94" s="16"/>
+      <c r="G94" s="17"/>
       <c r="H94" s="2"/>
     </row>
     <row r="95">
       <c r="A95" s="2"/>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 8</t>
-        </is>
-      </c>
-      <c r="C95" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The War's End</t>
-        </is>
-      </c>
-      <c r="D95" s="16"/>
-      <c r="E95" s="16"/>
-      <c r="F95" s="16"/>
-      <c r="G95" s="17"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D95" s="5"/>
+      <c r="E95" s="6"/>
+      <c r="F95" s="6"/>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L5 Emancipation and Life in Wartime</t>
+        </is>
+      </c>
       <c r="H95" s="2"/>
     </row>
     <row r="96">
       <c r="A96" s="2"/>
-      <c r="B96" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C96" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The War's End</t>
-        </is>
-      </c>
-      <c r="D96" s="5"/>
+      <c r="B96" s="4"/>
+      <c r="C96" s="5"/>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
-      <c r="G96" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L6 The War's End</t>
-        </is>
-      </c>
+      <c r="G96" s="6"/>
       <c r="H96" s="2"/>
     </row>
     <row r="97">
@@ -2086,7 +2146,7 @@
       <c r="C97" s="5"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E97" s="6"/>
@@ -2100,7 +2160,7 @@
       <c r="C98" s="5"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E98" s="6"/>
@@ -2114,7 +2174,7 @@
       <c r="C99" s="5"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E99" s="6"/>
@@ -2138,13 +2198,17 @@
     </row>
     <row r="101">
       <c r="A101" s="2"/>
-      <c r="B101" s="4"/>
-      <c r="C101" s="5"/>
-      <c r="D101" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D101" s="5"/>
       <c r="E101" s="6"/>
       <c r="F101" s="6"/>
       <c r="G101" s="6"/>
@@ -2152,70 +2216,66 @@
     </row>
     <row r="102">
       <c r="A102" s="2"/>
-      <c r="B102" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The War's End</t>
-        </is>
-      </c>
-      <c r="D102" s="5"/>
-      <c r="E102" s="6"/>
-      <c r="F102" s="6"/>
-      <c r="G102" s="6"/>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2"/>
+      <c r="D102" s="2"/>
+      <c r="E102" s="2"/>
+      <c r="F102" s="2"/>
+      <c r="G102" s="2"/>
       <c r="H102" s="2"/>
     </row>
     <row r="103">
       <c r="A103" s="2"/>
-      <c r="B103" s="2"/>
-      <c r="C103" s="2"/>
-      <c r="D103" s="2"/>
-      <c r="E103" s="2"/>
-      <c r="F103" s="2"/>
-      <c r="G103" s="2"/>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 8</t>
+        </is>
+      </c>
+      <c r="C103" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The War's End</t>
+        </is>
+      </c>
+      <c r="D103" s="16"/>
+      <c r="E103" s="16"/>
+      <c r="F103" s="16"/>
+      <c r="G103" s="17"/>
       <c r="H103" s="2"/>
     </row>
     <row r="104">
       <c r="A104" s="2"/>
-      <c r="B104" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 9</t>
-        </is>
-      </c>
-      <c r="C104" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D104" s="16"/>
-      <c r="E104" s="16"/>
-      <c r="F104" s="16"/>
-      <c r="G104" s="17"/>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The War's End</t>
+        </is>
+      </c>
+      <c r="D104" s="5"/>
+      <c r="E104" s="6"/>
+      <c r="F104" s="6"/>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L6 The War's End</t>
+        </is>
+      </c>
       <c r="H104" s="2"/>
     </row>
     <row r="105">
       <c r="A105" s="2"/>
-      <c r="B105" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D105" s="5"/>
+      <c r="B105" s="4"/>
+      <c r="C105" s="5"/>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
-      <c r="G105" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L1 Early Reconstruction; T7 L2 Radical Reconstruction</t>
-        </is>
-      </c>
+      <c r="G105" s="6"/>
       <c r="H105" s="2"/>
     </row>
     <row r="106">
@@ -2224,7 +2284,7 @@
       <c r="C106" s="5"/>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E106" s="6"/>
@@ -2238,7 +2298,7 @@
       <c r="C107" s="5"/>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E107" s="6"/>
@@ -2252,7 +2312,7 @@
       <c r="C108" s="5"/>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E108" s="6"/>
@@ -2276,13 +2336,17 @@
     </row>
     <row r="110">
       <c r="A110" s="2"/>
-      <c r="B110" s="4"/>
-      <c r="C110" s="5"/>
-      <c r="D110" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The War's End</t>
+        </is>
+      </c>
+      <c r="D110" s="5"/>
       <c r="E110" s="6"/>
       <c r="F110" s="6"/>
       <c r="G110" s="6"/>
@@ -2290,70 +2354,66 @@
     </row>
     <row r="111">
       <c r="A111" s="2"/>
-      <c r="B111" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D111" s="5"/>
-      <c r="E111" s="6"/>
-      <c r="F111" s="6"/>
-      <c r="G111" s="6"/>
+      <c r="B111" s="2"/>
+      <c r="C111" s="2"/>
+      <c r="D111" s="2"/>
+      <c r="E111" s="2"/>
+      <c r="F111" s="2"/>
+      <c r="G111" s="2"/>
       <c r="H111" s="2"/>
     </row>
     <row r="112">
       <c r="A112" s="2"/>
-      <c r="B112" s="2"/>
-      <c r="C112" s="2"/>
-      <c r="D112" s="2"/>
-      <c r="E112" s="2"/>
-      <c r="F112" s="2"/>
-      <c r="G112" s="2"/>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 9</t>
+        </is>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D112" s="16"/>
+      <c r="E112" s="16"/>
+      <c r="F112" s="16"/>
+      <c r="G112" s="17"/>
       <c r="H112" s="2"/>
     </row>
     <row r="113">
       <c r="A113" s="2"/>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 10</t>
-        </is>
-      </c>
-      <c r="C113" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D113" s="16"/>
-      <c r="E113" s="16"/>
-      <c r="F113" s="16"/>
-      <c r="G113" s="17"/>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D113" s="5"/>
+      <c r="E113" s="6"/>
+      <c r="F113" s="6"/>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T7 L1 Early Reconstruction; T7 L2 Radical Reconstruction</t>
+        </is>
+      </c>
       <c r="H113" s="2"/>
     </row>
     <row r="114">
       <c r="A114" s="2"/>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D114" s="5"/>
+      <c r="B114" s="4"/>
+      <c r="C114" s="5"/>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E114" s="6"/>
       <c r="F114" s="6"/>
-      <c r="G114" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L3 Reconstruction and Southern Society; T7 L4 The Aftermath of Reconstruction</t>
-        </is>
-      </c>
+      <c r="G114" s="6"/>
       <c r="H114" s="2"/>
     </row>
     <row r="115">
@@ -2362,7 +2422,7 @@
       <c r="C115" s="5"/>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E115" s="6"/>
@@ -2376,7 +2436,7 @@
       <c r="C116" s="5"/>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E116" s="6"/>
@@ -2390,7 +2450,7 @@
       <c r="C117" s="5"/>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E117" s="6"/>
@@ -2414,13 +2474,17 @@
     </row>
     <row r="119">
       <c r="A119" s="2"/>
-      <c r="B119" s="4"/>
-      <c r="C119" s="5"/>
-      <c r="D119" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D119" s="5"/>
       <c r="E119" s="6"/>
       <c r="F119" s="6"/>
       <c r="G119" s="6"/>
@@ -2428,63 +2492,63 @@
     </row>
     <row r="120">
       <c r="A120" s="2"/>
-      <c r="B120" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D120" s="5"/>
-      <c r="E120" s="6"/>
-      <c r="F120" s="6"/>
-      <c r="G120" s="6"/>
+      <c r="B120" s="2"/>
+      <c r="C120" s="2"/>
+      <c r="D120" s="2"/>
+      <c r="E120" s="2"/>
+      <c r="F120" s="2"/>
+      <c r="G120" s="2"/>
       <c r="H120" s="2"/>
     </row>
     <row r="121">
       <c r="A121" s="2"/>
-      <c r="B121" s="2"/>
-      <c r="C121" s="2"/>
-      <c r="D121" s="2"/>
-      <c r="E121" s="2"/>
-      <c r="F121" s="2"/>
-      <c r="G121" s="2"/>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 10</t>
+        </is>
+      </c>
+      <c r="C121" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D121" s="16"/>
+      <c r="E121" s="16"/>
+      <c r="F121" s="16"/>
+      <c r="G121" s="17"/>
       <c r="H121" s="2"/>
     </row>
     <row r="122">
       <c r="A122" s="2"/>
-      <c r="B122" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 11</t>
-        </is>
-      </c>
-      <c r="C122" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT — Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
-        </is>
-      </c>
-      <c r="D122" s="16"/>
-      <c r="E122" s="16"/>
-      <c r="F122" s="16"/>
-      <c r="G122" s="17"/>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D122" s="5"/>
+      <c r="E122" s="6"/>
+      <c r="F122" s="6"/>
+      <c r="G122" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T7 L3 Reconstruction and Southern Society; T7 L4 The Aftermath of Reconstruction</t>
+        </is>
+      </c>
       <c r="H122" s="2"/>
     </row>
     <row r="123">
       <c r="A123" s="2"/>
-      <c r="B123" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
-        </is>
-      </c>
-      <c r="D123" s="5"/>
+      <c r="B123" s="4"/>
+      <c r="C123" s="5"/>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E123" s="6"/>
       <c r="F123" s="6"/>
       <c r="G123" s="6"/>
@@ -2496,7 +2560,7 @@
       <c r="C124" s="5"/>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E124" s="6"/>
@@ -2506,17 +2570,13 @@
     </row>
     <row r="125">
       <c r="A125" s="2"/>
-      <c r="B125" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
-        </is>
-      </c>
-      <c r="D125" s="5"/>
+      <c r="B125" s="4"/>
+      <c r="C125" s="5"/>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E125" s="6"/>
       <c r="F125" s="6"/>
       <c r="G125" s="6"/>
@@ -2524,30 +2584,30 @@
     </row>
     <row r="126">
       <c r="A126" s="2"/>
-      <c r="B126" s="2"/>
-      <c r="C126" s="2"/>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2"/>
-      <c r="F126" s="2"/>
-      <c r="G126" s="2"/>
+      <c r="B126" s="4"/>
+      <c r="C126" s="5"/>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E126" s="6"/>
+      <c r="F126" s="6"/>
+      <c r="G126" s="6"/>
       <c r="H126" s="2"/>
     </row>
     <row r="127">
       <c r="A127" s="2"/>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 12</t>
-        </is>
-      </c>
-      <c r="C127" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D127" s="16"/>
-      <c r="E127" s="16"/>
-      <c r="F127" s="16"/>
-      <c r="G127" s="17"/>
+      <c r="B127" s="4"/>
+      <c r="C127" s="5"/>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E127" s="6"/>
+      <c r="F127" s="6"/>
+      <c r="G127" s="6"/>
       <c r="H127" s="2"/>
     </row>
     <row r="128">
@@ -2559,56 +2619,56 @@
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
+          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
         </is>
       </c>
       <c r="D128" s="5"/>
       <c r="E128" s="6"/>
       <c r="F128" s="6"/>
-      <c r="G128" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
-        </is>
-      </c>
+      <c r="G128" s="6"/>
       <c r="H128" s="2"/>
     </row>
     <row r="129">
       <c r="A129" s="2"/>
-      <c r="B129" s="4"/>
-      <c r="C129" s="5"/>
-      <c r="D129" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E129" s="6"/>
-      <c r="F129" s="6"/>
-      <c r="G129" s="6"/>
+      <c r="B129" s="2"/>
+      <c r="C129" s="2"/>
+      <c r="D129" s="2"/>
+      <c r="E129" s="2"/>
+      <c r="F129" s="2"/>
+      <c r="G129" s="2"/>
       <c r="H129" s="2"/>
     </row>
     <row r="130">
       <c r="A130" s="2"/>
-      <c r="B130" s="4"/>
-      <c r="C130" s="5"/>
-      <c r="D130" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E130" s="6"/>
-      <c r="F130" s="6"/>
-      <c r="G130" s="6"/>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 11</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT — Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
+        </is>
+      </c>
+      <c r="D130" s="16"/>
+      <c r="E130" s="16"/>
+      <c r="F130" s="16"/>
+      <c r="G130" s="17"/>
       <c r="H130" s="2"/>
     </row>
     <row r="131">
       <c r="A131" s="2"/>
-      <c r="B131" s="4"/>
-      <c r="C131" s="5"/>
-      <c r="D131" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
+        </is>
+      </c>
+      <c r="D131" s="5"/>
       <c r="E131" s="6"/>
       <c r="F131" s="6"/>
       <c r="G131" s="6"/>
@@ -2620,7 +2680,7 @@
       <c r="C132" s="5"/>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Custom project — detailed outline added when built</t>
         </is>
       </c>
       <c r="E132" s="6"/>
@@ -2630,13 +2690,17 @@
     </row>
     <row r="133">
       <c r="A133" s="2"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="5"/>
-      <c r="D133" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
+        </is>
+      </c>
+      <c r="D133" s="5"/>
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
       <c r="G133" s="6"/>
@@ -2644,70 +2708,66 @@
     </row>
     <row r="134">
       <c r="A134" s="2"/>
-      <c r="B134" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D134" s="5"/>
-      <c r="E134" s="6"/>
-      <c r="F134" s="6"/>
-      <c r="G134" s="6"/>
+      <c r="B134" s="2"/>
+      <c r="C134" s="2"/>
+      <c r="D134" s="2"/>
+      <c r="E134" s="2"/>
+      <c r="F134" s="2"/>
+      <c r="G134" s="2"/>
       <c r="H134" s="2"/>
     </row>
     <row r="135">
       <c r="A135" s="2"/>
-      <c r="B135" s="2"/>
-      <c r="C135" s="2"/>
-      <c r="D135" s="2"/>
-      <c r="E135" s="2"/>
-      <c r="F135" s="2"/>
-      <c r="G135" s="2"/>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 12</t>
+        </is>
+      </c>
+      <c r="C135" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
+        </is>
+      </c>
+      <c r="D135" s="16"/>
+      <c r="E135" s="16"/>
+      <c r="F135" s="16"/>
+      <c r="G135" s="17"/>
       <c r="H135" s="2"/>
     </row>
     <row r="136">
       <c r="A136" s="2"/>
-      <c r="B136" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 13</t>
-        </is>
-      </c>
-      <c r="C136" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D136" s="16"/>
-      <c r="E136" s="16"/>
-      <c r="F136" s="16"/>
-      <c r="G136" s="17"/>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
+        </is>
+      </c>
+      <c r="D136" s="5"/>
+      <c r="E136" s="6"/>
+      <c r="F136" s="6"/>
+      <c r="G136" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
+        </is>
+      </c>
       <c r="H136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D137" s="5"/>
+      <c r="B137" s="4"/>
+      <c r="C137" s="5"/>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
-      <c r="G137" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
-        </is>
-      </c>
+      <c r="G137" s="6"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138">
@@ -2716,7 +2776,7 @@
       <c r="C138" s="5"/>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E138" s="6"/>
@@ -2730,7 +2790,7 @@
       <c r="C139" s="5"/>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E139" s="6"/>
@@ -2744,7 +2804,7 @@
       <c r="C140" s="5"/>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E140" s="6"/>
@@ -2768,13 +2828,17 @@
     </row>
     <row r="142">
       <c r="A142" s="2"/>
-      <c r="B142" s="4"/>
-      <c r="C142" s="5"/>
-      <c r="D142" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
+        </is>
+      </c>
+      <c r="D142" s="5"/>
       <c r="E142" s="6"/>
       <c r="F142" s="6"/>
       <c r="G142" s="6"/>
@@ -2782,70 +2846,66 @@
     </row>
     <row r="143">
       <c r="A143" s="2"/>
-      <c r="B143" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D143" s="5"/>
-      <c r="E143" s="6"/>
-      <c r="F143" s="6"/>
-      <c r="G143" s="6"/>
+      <c r="B143" s="2"/>
+      <c r="C143" s="2"/>
+      <c r="D143" s="2"/>
+      <c r="E143" s="2"/>
+      <c r="F143" s="2"/>
+      <c r="G143" s="2"/>
       <c r="H143" s="2"/>
     </row>
     <row r="144">
       <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
-      <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
-      <c r="F144" s="2"/>
-      <c r="G144" s="2"/>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 13</t>
+        </is>
+      </c>
+      <c r="C144" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D144" s="16"/>
+      <c r="E144" s="16"/>
+      <c r="F144" s="16"/>
+      <c r="G144" s="17"/>
       <c r="H144" s="2"/>
     </row>
     <row r="145">
       <c r="A145" s="2"/>
-      <c r="B145" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 14</t>
-        </is>
-      </c>
-      <c r="C145" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D145" s="16"/>
-      <c r="E145" s="16"/>
-      <c r="F145" s="16"/>
-      <c r="G145" s="17"/>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D145" s="5"/>
+      <c r="E145" s="6"/>
+      <c r="F145" s="6"/>
+      <c r="G145" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
+        </is>
+      </c>
       <c r="H145" s="2"/>
     </row>
     <row r="146">
       <c r="A146" s="2"/>
-      <c r="B146" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D146" s="5"/>
+      <c r="B146" s="4"/>
+      <c r="C146" s="5"/>
+      <c r="D146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
-      <c r="G146" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
-        </is>
-      </c>
+      <c r="G146" s="6"/>
       <c r="H146" s="2"/>
     </row>
     <row r="147">
@@ -2854,7 +2914,7 @@
       <c r="C147" s="5"/>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E147" s="6"/>
@@ -2868,7 +2928,7 @@
       <c r="C148" s="5"/>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E148" s="6"/>
@@ -2882,7 +2942,7 @@
       <c r="C149" s="5"/>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E149" s="6"/>
@@ -2906,13 +2966,17 @@
     </row>
     <row r="151">
       <c r="A151" s="2"/>
-      <c r="B151" s="4"/>
-      <c r="C151" s="5"/>
-      <c r="D151" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D151" s="5"/>
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
       <c r="G151" s="6"/>
@@ -2920,70 +2984,66 @@
     </row>
     <row r="152">
       <c r="A152" s="2"/>
-      <c r="B152" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C152" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D152" s="5"/>
-      <c r="E152" s="6"/>
-      <c r="F152" s="6"/>
-      <c r="G152" s="6"/>
+      <c r="B152" s="2"/>
+      <c r="C152" s="2"/>
+      <c r="D152" s="2"/>
+      <c r="E152" s="2"/>
+      <c r="F152" s="2"/>
+      <c r="G152" s="2"/>
       <c r="H152" s="2"/>
     </row>
     <row r="153">
       <c r="A153" s="2"/>
-      <c r="B153" s="2"/>
-      <c r="C153" s="2"/>
-      <c r="D153" s="2"/>
-      <c r="E153" s="2"/>
-      <c r="F153" s="2"/>
-      <c r="G153" s="2"/>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 14</t>
+        </is>
+      </c>
+      <c r="C153" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="D153" s="16"/>
+      <c r="E153" s="16"/>
+      <c r="F153" s="16"/>
+      <c r="G153" s="17"/>
       <c r="H153" s="2"/>
     </row>
     <row r="154">
       <c r="A154" s="2"/>
-      <c r="B154" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 15</t>
-        </is>
-      </c>
-      <c r="C154" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New Technologies</t>
-        </is>
-      </c>
-      <c r="D154" s="16"/>
-      <c r="E154" s="16"/>
-      <c r="F154" s="16"/>
-      <c r="G154" s="17"/>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="D154" s="5"/>
+      <c r="E154" s="6"/>
+      <c r="F154" s="6"/>
+      <c r="G154" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
+        </is>
+      </c>
       <c r="H154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2"/>
-      <c r="B155" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | New Technologies</t>
-        </is>
-      </c>
-      <c r="D155" s="5"/>
+      <c r="B155" s="4"/>
+      <c r="C155" s="5"/>
+      <c r="D155" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
-      <c r="G155" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
-        </is>
-      </c>
+      <c r="G155" s="6"/>
       <c r="H155" s="2"/>
     </row>
     <row r="156">
@@ -2992,7 +3052,7 @@
       <c r="C156" s="5"/>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E156" s="6"/>
@@ -3006,7 +3066,7 @@
       <c r="C157" s="5"/>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E157" s="6"/>
@@ -3020,7 +3080,7 @@
       <c r="C158" s="5"/>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E158" s="6"/>
@@ -3044,13 +3104,17 @@
     </row>
     <row r="160">
       <c r="A160" s="2"/>
-      <c r="B160" s="4"/>
-      <c r="C160" s="5"/>
-      <c r="D160" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="D160" s="5"/>
       <c r="E160" s="6"/>
       <c r="F160" s="6"/>
       <c r="G160" s="6"/>
@@ -3058,70 +3122,66 @@
     </row>
     <row r="161">
       <c r="A161" s="2"/>
-      <c r="B161" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C161" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | New Technologies</t>
-        </is>
-      </c>
-      <c r="D161" s="5"/>
-      <c r="E161" s="6"/>
-      <c r="F161" s="6"/>
-      <c r="G161" s="6"/>
+      <c r="B161" s="2"/>
+      <c r="C161" s="2"/>
+      <c r="D161" s="2"/>
+      <c r="E161" s="2"/>
+      <c r="F161" s="2"/>
+      <c r="G161" s="2"/>
       <c r="H161" s="2"/>
     </row>
     <row r="162">
       <c r="A162" s="2"/>
-      <c r="B162" s="2"/>
-      <c r="C162" s="2"/>
-      <c r="D162" s="2"/>
-      <c r="E162" s="2"/>
-      <c r="F162" s="2"/>
-      <c r="G162" s="2"/>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 15</t>
+        </is>
+      </c>
+      <c r="C162" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Technologies</t>
+        </is>
+      </c>
+      <c r="D162" s="16"/>
+      <c r="E162" s="16"/>
+      <c r="F162" s="16"/>
+      <c r="G162" s="17"/>
       <c r="H162" s="2"/>
     </row>
     <row r="163">
       <c r="A163" s="2"/>
-      <c r="B163" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 16</t>
-        </is>
-      </c>
-      <c r="C163" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D163" s="16"/>
-      <c r="E163" s="16"/>
-      <c r="F163" s="16"/>
-      <c r="G163" s="17"/>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | New Technologies</t>
+        </is>
+      </c>
+      <c r="D163" s="5"/>
+      <c r="E163" s="6"/>
+      <c r="F163" s="6"/>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
+        </is>
+      </c>
       <c r="H163" s="2"/>
     </row>
     <row r="164">
       <c r="A164" s="2"/>
-      <c r="B164" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C164" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D164" s="5"/>
+      <c r="B164" s="4"/>
+      <c r="C164" s="5"/>
+      <c r="D164" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E164" s="6"/>
       <c r="F164" s="6"/>
-      <c r="G164" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
-        </is>
-      </c>
+      <c r="G164" s="6"/>
       <c r="H164" s="2"/>
     </row>
     <row r="165">
@@ -3130,7 +3190,7 @@
       <c r="C165" s="5"/>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E165" s="6"/>
@@ -3144,7 +3204,7 @@
       <c r="C166" s="5"/>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E166" s="6"/>
@@ -3158,7 +3218,7 @@
       <c r="C167" s="5"/>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E167" s="6"/>
@@ -3182,13 +3242,17 @@
     </row>
     <row r="169">
       <c r="A169" s="2"/>
-      <c r="B169" s="4"/>
-      <c r="C169" s="5"/>
-      <c r="D169" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | New Technologies</t>
+        </is>
+      </c>
+      <c r="D169" s="5"/>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
@@ -3196,70 +3260,66 @@
     </row>
     <row r="170">
       <c r="A170" s="2"/>
-      <c r="B170" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C170" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D170" s="5"/>
-      <c r="E170" s="6"/>
-      <c r="F170" s="6"/>
-      <c r="G170" s="6"/>
+      <c r="B170" s="2"/>
+      <c r="C170" s="2"/>
+      <c r="D170" s="2"/>
+      <c r="E170" s="2"/>
+      <c r="F170" s="2"/>
+      <c r="G170" s="2"/>
       <c r="H170" s="2"/>
     </row>
     <row r="171">
       <c r="A171" s="2"/>
-      <c r="B171" s="2"/>
-      <c r="C171" s="2"/>
-      <c r="D171" s="2"/>
-      <c r="E171" s="2"/>
-      <c r="F171" s="2"/>
-      <c r="G171" s="2"/>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 16</t>
+        </is>
+      </c>
+      <c r="C171" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D171" s="16"/>
+      <c r="E171" s="16"/>
+      <c r="F171" s="16"/>
+      <c r="G171" s="17"/>
       <c r="H171" s="2"/>
     </row>
     <row r="172">
       <c r="A172" s="2"/>
-      <c r="B172" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 17</t>
-        </is>
-      </c>
-      <c r="C172" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Progressive Movement</t>
-        </is>
-      </c>
-      <c r="D172" s="16"/>
-      <c r="E172" s="16"/>
-      <c r="F172" s="16"/>
-      <c r="G172" s="17"/>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D172" s="5"/>
+      <c r="E172" s="6"/>
+      <c r="F172" s="6"/>
+      <c r="G172" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
+        </is>
+      </c>
       <c r="H172" s="2"/>
     </row>
     <row r="173">
       <c r="A173" s="2"/>
-      <c r="B173" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C173" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Progressive Movement</t>
-        </is>
-      </c>
-      <c r="D173" s="5"/>
+      <c r="B173" s="4"/>
+      <c r="C173" s="5"/>
+      <c r="D173" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
-      <c r="G173" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
-        </is>
-      </c>
+      <c r="G173" s="6"/>
       <c r="H173" s="2"/>
     </row>
     <row r="174">
@@ -3268,7 +3328,7 @@
       <c r="C174" s="5"/>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E174" s="6"/>
@@ -3282,7 +3342,7 @@
       <c r="C175" s="5"/>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E175" s="6"/>
@@ -3296,7 +3356,7 @@
       <c r="C176" s="5"/>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E176" s="6"/>
@@ -3320,13 +3380,17 @@
     </row>
     <row r="178">
       <c r="A178" s="2"/>
-      <c r="B178" s="4"/>
-      <c r="C178" s="5"/>
-      <c r="D178" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C178" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D178" s="5"/>
       <c r="E178" s="6"/>
       <c r="F178" s="6"/>
       <c r="G178" s="6"/>
@@ -3334,70 +3398,66 @@
     </row>
     <row r="179">
       <c r="A179" s="2"/>
-      <c r="B179" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C179" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
-        </is>
-      </c>
-      <c r="D179" s="5"/>
-      <c r="E179" s="6"/>
-      <c r="F179" s="6"/>
-      <c r="G179" s="6"/>
+      <c r="B179" s="2"/>
+      <c r="C179" s="2"/>
+      <c r="D179" s="2"/>
+      <c r="E179" s="2"/>
+      <c r="F179" s="2"/>
+      <c r="G179" s="2"/>
       <c r="H179" s="2"/>
     </row>
     <row r="180">
       <c r="A180" s="2"/>
-      <c r="B180" s="2"/>
-      <c r="C180" s="2"/>
-      <c r="D180" s="2"/>
-      <c r="E180" s="2"/>
-      <c r="F180" s="2"/>
-      <c r="G180" s="2"/>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 17</t>
+        </is>
+      </c>
+      <c r="C180" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D180" s="16"/>
+      <c r="E180" s="16"/>
+      <c r="F180" s="16"/>
+      <c r="G180" s="17"/>
       <c r="H180" s="2"/>
     </row>
     <row r="181">
       <c r="A181" s="2"/>
-      <c r="B181" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 18</t>
-        </is>
-      </c>
-      <c r="C181" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
-        </is>
-      </c>
-      <c r="D181" s="16"/>
-      <c r="E181" s="16"/>
-      <c r="F181" s="16"/>
-      <c r="G181" s="17"/>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C181" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D181" s="5"/>
+      <c r="E181" s="6"/>
+      <c r="F181" s="6"/>
+      <c r="G181" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
+        </is>
+      </c>
       <c r="H181" s="2"/>
     </row>
     <row r="182">
       <c r="A182" s="2"/>
-      <c r="B182" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C182" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
-        </is>
-      </c>
-      <c r="D182" s="5"/>
+      <c r="B182" s="4"/>
+      <c r="C182" s="5"/>
+      <c r="D182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E182" s="6"/>
       <c r="F182" s="6"/>
-      <c r="G182" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
-        </is>
-      </c>
+      <c r="G182" s="6"/>
       <c r="H182" s="2"/>
     </row>
     <row r="183">
@@ -3406,7 +3466,7 @@
       <c r="C183" s="5"/>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E183" s="6"/>
@@ -3420,7 +3480,7 @@
       <c r="C184" s="5"/>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E184" s="6"/>
@@ -3434,7 +3494,7 @@
       <c r="C185" s="5"/>
       <c r="D185" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E185" s="6"/>
@@ -3458,13 +3518,17 @@
     </row>
     <row r="187">
       <c r="A187" s="2"/>
-      <c r="B187" s="4"/>
-      <c r="C187" s="5"/>
-      <c r="D187" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D187" s="5"/>
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
@@ -3472,63 +3536,63 @@
     </row>
     <row r="188">
       <c r="A188" s="2"/>
-      <c r="B188" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C188" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
-        </is>
-      </c>
-      <c r="D188" s="5"/>
-      <c r="E188" s="6"/>
-      <c r="F188" s="6"/>
-      <c r="G188" s="6"/>
+      <c r="B188" s="2"/>
+      <c r="C188" s="2"/>
+      <c r="D188" s="2"/>
+      <c r="E188" s="2"/>
+      <c r="F188" s="2"/>
+      <c r="G188" s="2"/>
       <c r="H188" s="2"/>
     </row>
     <row r="189">
       <c r="A189" s="2"/>
-      <c r="B189" s="2"/>
-      <c r="C189" s="2"/>
-      <c r="D189" s="2"/>
-      <c r="E189" s="2"/>
-      <c r="F189" s="2"/>
-      <c r="G189" s="2"/>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 18</t>
+        </is>
+      </c>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D189" s="16"/>
+      <c r="E189" s="16"/>
+      <c r="F189" s="16"/>
+      <c r="G189" s="17"/>
       <c r="H189" s="2"/>
     </row>
     <row r="190">
       <c r="A190" s="2"/>
-      <c r="B190" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 19</t>
-        </is>
-      </c>
-      <c r="C190" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
-        </is>
-      </c>
-      <c r="D190" s="16"/>
-      <c r="E190" s="16"/>
-      <c r="F190" s="16"/>
-      <c r="G190" s="17"/>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C190" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D190" s="5"/>
+      <c r="E190" s="6"/>
+      <c r="F190" s="6"/>
+      <c r="G190" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
+        </is>
+      </c>
       <c r="H190" s="2"/>
     </row>
     <row r="191">
       <c r="A191" s="2"/>
-      <c r="B191" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C191" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D191" s="5"/>
+      <c r="B191" s="4"/>
+      <c r="C191" s="5"/>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
       <c r="G191" s="6"/>
@@ -3540,7 +3604,7 @@
       <c r="C192" s="5"/>
       <c r="D192" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E192" s="6"/>
@@ -3550,17 +3614,13 @@
     </row>
     <row r="193">
       <c r="A193" s="2"/>
-      <c r="B193" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C193" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D193" s="5"/>
+      <c r="B193" s="4"/>
+      <c r="C193" s="5"/>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
       <c r="G193" s="6"/>
@@ -3568,30 +3628,30 @@
     </row>
     <row r="194">
       <c r="A194" s="2"/>
-      <c r="B194" s="2"/>
-      <c r="C194" s="2"/>
-      <c r="D194" s="2"/>
-      <c r="E194" s="2"/>
-      <c r="F194" s="2"/>
-      <c r="G194" s="2"/>
+      <c r="B194" s="4"/>
+      <c r="C194" s="5"/>
+      <c r="D194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E194" s="6"/>
+      <c r="F194" s="6"/>
+      <c r="G194" s="6"/>
       <c r="H194" s="2"/>
     </row>
     <row r="195">
       <c r="A195" s="2"/>
-      <c r="B195" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C195" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D195" s="16"/>
-      <c r="E195" s="16"/>
-      <c r="F195" s="16"/>
-      <c r="G195" s="17"/>
+      <c r="B195" s="4"/>
+      <c r="C195" s="5"/>
+      <c r="D195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E195" s="6"/>
+      <c r="F195" s="6"/>
+      <c r="G195" s="6"/>
       <c r="H195" s="2"/>
     </row>
     <row r="196">
@@ -3603,7 +3663,7 @@
       </c>
       <c r="C196" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Final Exam</t>
+          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
         </is>
       </c>
       <c r="D196" s="5"/>
@@ -3614,41 +3674,45 @@
     </row>
     <row r="197">
       <c r="A197" s="2"/>
-      <c r="B197" s="4"/>
-      <c r="C197" s="5"/>
-      <c r="D197" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E197" s="6"/>
-      <c r="F197" s="6"/>
-      <c r="G197" s="6"/>
+      <c r="B197" s="2"/>
+      <c r="C197" s="2"/>
+      <c r="D197" s="2"/>
+      <c r="E197" s="2"/>
+      <c r="F197" s="2"/>
+      <c r="G197" s="2"/>
       <c r="H197" s="2"/>
     </row>
     <row r="198">
       <c r="A198" s="2"/>
-      <c r="B198" s="4"/>
-      <c r="C198" s="5"/>
-      <c r="D198" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E198" s="6"/>
-      <c r="F198" s="6"/>
-      <c r="G198" s="6"/>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C198" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D198" s="16"/>
+      <c r="E198" s="16"/>
+      <c r="F198" s="16"/>
+      <c r="G198" s="17"/>
       <c r="H198" s="2"/>
     </row>
     <row r="199">
       <c r="A199" s="2"/>
-      <c r="B199" s="4"/>
-      <c r="C199" s="5"/>
-      <c r="D199" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C199" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D199" s="5"/>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
       <c r="G199" s="6"/>
@@ -3660,7 +3724,7 @@
       <c r="C200" s="5"/>
       <c r="D200" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Custom project — detailed outline added when built</t>
         </is>
       </c>
       <c r="E200" s="6"/>
@@ -3670,13 +3734,17 @@
     </row>
     <row r="201">
       <c r="A201" s="2"/>
-      <c r="B201" s="4"/>
-      <c r="C201" s="5"/>
-      <c r="D201" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C201" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D201" s="5"/>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
       <c r="G201" s="6"/>
@@ -3684,31 +3752,147 @@
     </row>
     <row r="202">
       <c r="A202" s="2"/>
-      <c r="B202" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C202" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Final Exam</t>
-        </is>
-      </c>
-      <c r="D202" s="5"/>
-      <c r="E202" s="6"/>
-      <c r="F202" s="6"/>
-      <c r="G202" s="6"/>
+      <c r="B202" s="2"/>
+      <c r="C202" s="2"/>
+      <c r="D202" s="2"/>
+      <c r="E202" s="2"/>
+      <c r="F202" s="2"/>
+      <c r="G202" s="2"/>
       <c r="H202" s="2"/>
     </row>
     <row r="203">
       <c r="A203" s="2"/>
-      <c r="B203" s="2"/>
-      <c r="C203" s="2"/>
-      <c r="D203" s="2"/>
-      <c r="E203" s="2"/>
-      <c r="F203" s="2"/>
-      <c r="G203" s="2"/>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C203" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D203" s="16"/>
+      <c r="E203" s="16"/>
+      <c r="F203" s="16"/>
+      <c r="G203" s="17"/>
       <c r="H203" s="2"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="2"/>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C204" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Final Exam</t>
+        </is>
+      </c>
+      <c r="D204" s="5"/>
+      <c r="E204" s="6"/>
+      <c r="F204" s="6"/>
+      <c r="G204" s="6"/>
+      <c r="H204" s="2"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="2"/>
+      <c r="B205" s="4"/>
+      <c r="C205" s="5"/>
+      <c r="D205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E205" s="6"/>
+      <c r="F205" s="6"/>
+      <c r="G205" s="6"/>
+      <c r="H205" s="2"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="2"/>
+      <c r="B206" s="4"/>
+      <c r="C206" s="5"/>
+      <c r="D206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E206" s="6"/>
+      <c r="F206" s="6"/>
+      <c r="G206" s="6"/>
+      <c r="H206" s="2"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="2"/>
+      <c r="B207" s="4"/>
+      <c r="C207" s="5"/>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E207" s="6"/>
+      <c r="F207" s="6"/>
+      <c r="G207" s="6"/>
+      <c r="H207" s="2"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="2"/>
+      <c r="B208" s="4"/>
+      <c r="C208" s="5"/>
+      <c r="D208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E208" s="6"/>
+      <c r="F208" s="6"/>
+      <c r="G208" s="6"/>
+      <c r="H208" s="2"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="2"/>
+      <c r="B209" s="4"/>
+      <c r="C209" s="5"/>
+      <c r="D209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E209" s="6"/>
+      <c r="F209" s="6"/>
+      <c r="G209" s="6"/>
+      <c r="H209" s="2"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="2"/>
+      <c r="B210" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C210" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Final Exam</t>
+        </is>
+      </c>
+      <c r="D210" s="5"/>
+      <c r="E210" s="6"/>
+      <c r="F210" s="6"/>
+      <c r="G210" s="6"/>
+      <c r="H210" s="2"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="2"/>
+      <c r="B211" s="2"/>
+      <c r="C211" s="2"/>
+      <c r="D211" s="2"/>
+      <c r="E211" s="2"/>
+      <c r="F211" s="2"/>
+      <c r="G211" s="2"/>
+      <c r="H211" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -3718,22 +3902,22 @@
     <mergeCell ref="C30:G30"/>
     <mergeCell ref="C45:G45"/>
     <mergeCell ref="C59:G59"/>
-    <mergeCell ref="C68:G68"/>
-    <mergeCell ref="C77:G77"/>
-    <mergeCell ref="C86:G86"/>
-    <mergeCell ref="C95:G95"/>
-    <mergeCell ref="C104:G104"/>
-    <mergeCell ref="C113:G113"/>
-    <mergeCell ref="C122:G122"/>
-    <mergeCell ref="C127:G127"/>
-    <mergeCell ref="C136:G136"/>
-    <mergeCell ref="C145:G145"/>
-    <mergeCell ref="C154:G154"/>
-    <mergeCell ref="C163:G163"/>
-    <mergeCell ref="C172:G172"/>
-    <mergeCell ref="C181:G181"/>
-    <mergeCell ref="C190:G190"/>
-    <mergeCell ref="C195:G195"/>
+    <mergeCell ref="C76:G76"/>
+    <mergeCell ref="C85:G85"/>
+    <mergeCell ref="C94:G94"/>
+    <mergeCell ref="C103:G103"/>
+    <mergeCell ref="C112:G112"/>
+    <mergeCell ref="C121:G121"/>
+    <mergeCell ref="C130:G130"/>
+    <mergeCell ref="C135:G135"/>
+    <mergeCell ref="C144:G144"/>
+    <mergeCell ref="C153:G153"/>
+    <mergeCell ref="C162:G162"/>
+    <mergeCell ref="C171:G171"/>
+    <mergeCell ref="C180:G180"/>
+    <mergeCell ref="C189:G189"/>
+    <mergeCell ref="C198:G198"/>
+    <mergeCell ref="C203:G203"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add US History 8-2 Module 5 to dashboard
</commit_message>
<xml_diff>
--- a/exports/US History 8-2 - Course Outline.xlsx
+++ b/exports/US History 8-2 - Course Outline.xlsx
@@ -1842,17 +1842,25 @@
       </c>
       <c r="D77" s="5"/>
       <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.9.4, 8.9.5, 8.9.6, 8.10.1, 8.10.2 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.8, W.8.1, W.8.9 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T6 L1 Conflicts and Compromises; T6 L2 Growing Tensions</t>
+          <t xml:space="preserve">Why did compromises over slavery fail to stop sectional conflict from pushing the United States toward civil war?</t>
         </is>
       </c>
       <c r="H77" s="2"/>
     </row>
     <row r="78">
       <c r="A78" s="2"/>
-      <c r="B78" s="4"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C78" s="5"/>
       <c r="D78" s="7" t="inlineStr">
         <is>
@@ -1866,11 +1874,15 @@
     </row>
     <row r="79">
       <c r="A79" s="2"/>
-      <c r="B79" s="4"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C79" s="5"/>
-      <c r="D79" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Conflicts and Compromises</t>
         </is>
       </c>
       <c r="E79" s="6"/>
@@ -1880,11 +1892,15 @@
     </row>
     <row r="80">
       <c r="A80" s="2"/>
-      <c r="B80" s="4"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C80" s="5"/>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Growing Tensions</t>
         </is>
       </c>
       <c r="E80" s="6"/>
@@ -1894,25 +1910,37 @@
     </row>
     <row r="81">
       <c r="A81" s="2"/>
-      <c r="B81" s="4"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C81" s="5"/>
-      <c r="D81" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Compromise and Growing Tensions</t>
         </is>
       </c>
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
-      <c r="G81" s="6"/>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H81" s="2"/>
     </row>
     <row r="82">
       <c r="A82" s="2"/>
-      <c r="B82" s="4"/>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C82" s="5"/>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E82" s="6"/>
@@ -1924,15 +1952,15 @@
       <c r="A83" s="2"/>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
-        </is>
-      </c>
-      <c r="D83" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C83" s="5"/>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Cartoon: The Fugitive Slave Act</t>
+        </is>
+      </c>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
       <c r="G83" s="6"/>
@@ -1940,75 +1968,95 @@
     </row>
     <row r="84">
       <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="2"/>
-      <c r="G84" s="2"/>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C84" s="5"/>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: The Effects of the Kansas-Nebraska Act</t>
+        </is>
+      </c>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
+      <c r="G84" s="6"/>
       <c r="H84" s="2"/>
     </row>
     <row r="85">
       <c r="A85" s="2"/>
-      <c r="B85" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 6</t>
-        </is>
-      </c>
-      <c r="C85" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D85" s="16"/>
-      <c r="E85" s="16"/>
-      <c r="F85" s="16"/>
-      <c r="G85" s="17"/>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C85" s="5"/>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5.3.3 | DBQ: Lincoln &amp; Douglas</t>
+        </is>
+      </c>
+      <c r="E85" s="6"/>
+      <c r="F85" s="6"/>
+      <c r="G85" s="6"/>
       <c r="H85" s="2"/>
     </row>
     <row r="86">
       <c r="A86" s="2"/>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D86" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C86" s="5"/>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
+        </is>
+      </c>
       <c r="E86" s="6"/>
       <c r="F86" s="6"/>
       <c r="G86" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T6 L3 Division and the Outbreak of War; T6 L4 The Course of the War</t>
+          <t xml:space="preserve">6 questions</t>
         </is>
       </c>
       <c r="H86" s="2"/>
     </row>
     <row r="87">
       <c r="A87" s="2"/>
-      <c r="B87" s="4"/>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C87" s="5"/>
-      <c r="D87" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Law That Tried to Turn Everyone Into a Slave Catcher</t>
         </is>
       </c>
       <c r="E87" s="6"/>
       <c r="F87" s="6"/>
-      <c r="G87" s="6"/>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H87" s="2"/>
     </row>
     <row r="88">
       <c r="A88" s="2"/>
-      <c r="B88" s="4"/>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C88" s="5"/>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E88" s="6"/>
@@ -2018,27 +2066,39 @@
     </row>
     <row r="89">
       <c r="A89" s="2"/>
-      <c r="B89" s="4"/>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C89" s="5"/>
-      <c r="D89" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
         </is>
       </c>
       <c r="E89" s="6"/>
       <c r="F89" s="6"/>
-      <c r="G89" s="6"/>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H89" s="2"/>
     </row>
     <row r="90">
       <c r="A90" s="2"/>
-      <c r="B90" s="4"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Road to War: Compromises &amp; Tensions (+ DBQ: Lincoln &amp; Douglas)</t>
+        </is>
+      </c>
+      <c r="D90" s="5"/>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
       <c r="G90" s="6"/>
@@ -2046,84 +2106,80 @@
     </row>
     <row r="91">
       <c r="A91" s="2"/>
-      <c r="B91" s="4"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E91" s="6"/>
-      <c r="F91" s="6"/>
-      <c r="G91" s="6"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
       <c r="H91" s="2"/>
     </row>
     <row r="92">
       <c r="A92" s="2"/>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C92" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D92" s="5"/>
-      <c r="E92" s="6"/>
-      <c r="F92" s="6"/>
-      <c r="G92" s="6"/>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 6</t>
+        </is>
+      </c>
+      <c r="C92" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D92" s="16"/>
+      <c r="E92" s="16"/>
+      <c r="F92" s="16"/>
+      <c r="G92" s="17"/>
       <c r="H92" s="2"/>
     </row>
     <row r="93">
       <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="2"/>
-      <c r="G93" s="2"/>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D93" s="5"/>
+      <c r="E93" s="6"/>
+      <c r="F93" s="6"/>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L3 Division and the Outbreak of War; T6 L4 The Course of the War</t>
+        </is>
+      </c>
       <c r="H93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 7</t>
-        </is>
-      </c>
-      <c r="C94" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D94" s="16"/>
-      <c r="E94" s="16"/>
-      <c r="F94" s="16"/>
-      <c r="G94" s="17"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="5"/>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E94" s="6"/>
+      <c r="F94" s="6"/>
+      <c r="G94" s="6"/>
       <c r="H94" s="2"/>
     </row>
     <row r="95">
       <c r="A95" s="2"/>
-      <c r="B95" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D95" s="5"/>
+      <c r="B95" s="4"/>
+      <c r="C95" s="5"/>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
-      <c r="G95" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L5 Emancipation and Life in Wartime</t>
-        </is>
-      </c>
+      <c r="G95" s="6"/>
       <c r="H95" s="2"/>
     </row>
     <row r="96">
@@ -2132,7 +2188,7 @@
       <c r="C96" s="5"/>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E96" s="6"/>
@@ -2146,7 +2202,7 @@
       <c r="C97" s="5"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E97" s="6"/>
@@ -2160,7 +2216,7 @@
       <c r="C98" s="5"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E98" s="6"/>
@@ -2170,13 +2226,17 @@
     </row>
     <row r="99">
       <c r="A99" s="2"/>
-      <c r="B99" s="4"/>
-      <c r="C99" s="5"/>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D99" s="5"/>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
       <c r="G99" s="6"/>
@@ -2184,84 +2244,80 @@
     </row>
     <row r="100">
       <c r="A100" s="2"/>
-      <c r="B100" s="4"/>
-      <c r="C100" s="5"/>
-      <c r="D100" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E100" s="6"/>
-      <c r="F100" s="6"/>
-      <c r="G100" s="6"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
       <c r="H100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2"/>
-      <c r="B101" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D101" s="5"/>
-      <c r="E101" s="6"/>
-      <c r="F101" s="6"/>
-      <c r="G101" s="6"/>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 7</t>
+        </is>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D101" s="16"/>
+      <c r="E101" s="16"/>
+      <c r="F101" s="16"/>
+      <c r="G101" s="17"/>
       <c r="H101" s="2"/>
     </row>
     <row r="102">
       <c r="A102" s="2"/>
-      <c r="B102" s="2"/>
-      <c r="C102" s="2"/>
-      <c r="D102" s="2"/>
-      <c r="E102" s="2"/>
-      <c r="F102" s="2"/>
-      <c r="G102" s="2"/>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D102" s="5"/>
+      <c r="E102" s="6"/>
+      <c r="F102" s="6"/>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L5 Emancipation and Life in Wartime</t>
+        </is>
+      </c>
       <c r="H102" s="2"/>
     </row>
     <row r="103">
       <c r="A103" s="2"/>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 8</t>
-        </is>
-      </c>
-      <c r="C103" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The War's End</t>
-        </is>
-      </c>
-      <c r="D103" s="16"/>
-      <c r="E103" s="16"/>
-      <c r="F103" s="16"/>
-      <c r="G103" s="17"/>
+      <c r="B103" s="4"/>
+      <c r="C103" s="5"/>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E103" s="6"/>
+      <c r="F103" s="6"/>
+      <c r="G103" s="6"/>
       <c r="H103" s="2"/>
     </row>
     <row r="104">
       <c r="A104" s="2"/>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The War's End</t>
-        </is>
-      </c>
-      <c r="D104" s="5"/>
+      <c r="B104" s="4"/>
+      <c r="C104" s="5"/>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L6 The War's End</t>
-        </is>
-      </c>
+      <c r="G104" s="6"/>
       <c r="H104" s="2"/>
     </row>
     <row r="105">
@@ -2270,7 +2326,7 @@
       <c r="C105" s="5"/>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E105" s="6"/>
@@ -2284,7 +2340,7 @@
       <c r="C106" s="5"/>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E106" s="6"/>
@@ -2298,7 +2354,7 @@
       <c r="C107" s="5"/>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E107" s="6"/>
@@ -2308,13 +2364,17 @@
     </row>
     <row r="108">
       <c r="A108" s="2"/>
-      <c r="B108" s="4"/>
-      <c r="C108" s="5"/>
-      <c r="D108" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D108" s="5"/>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
       <c r="G108" s="6"/>
@@ -2322,84 +2382,80 @@
     </row>
     <row r="109">
       <c r="A109" s="2"/>
-      <c r="B109" s="4"/>
-      <c r="C109" s="5"/>
-      <c r="D109" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E109" s="6"/>
-      <c r="F109" s="6"/>
-      <c r="G109" s="6"/>
+      <c r="B109" s="2"/>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2"/>
+      <c r="E109" s="2"/>
+      <c r="F109" s="2"/>
+      <c r="G109" s="2"/>
       <c r="H109" s="2"/>
     </row>
     <row r="110">
       <c r="A110" s="2"/>
-      <c r="B110" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The War's End</t>
-        </is>
-      </c>
-      <c r="D110" s="5"/>
-      <c r="E110" s="6"/>
-      <c r="F110" s="6"/>
-      <c r="G110" s="6"/>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 8</t>
+        </is>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The War's End</t>
+        </is>
+      </c>
+      <c r="D110" s="16"/>
+      <c r="E110" s="16"/>
+      <c r="F110" s="16"/>
+      <c r="G110" s="17"/>
       <c r="H110" s="2"/>
     </row>
     <row r="111">
       <c r="A111" s="2"/>
-      <c r="B111" s="2"/>
-      <c r="C111" s="2"/>
-      <c r="D111" s="2"/>
-      <c r="E111" s="2"/>
-      <c r="F111" s="2"/>
-      <c r="G111" s="2"/>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The War's End</t>
+        </is>
+      </c>
+      <c r="D111" s="5"/>
+      <c r="E111" s="6"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T6 L6 The War's End</t>
+        </is>
+      </c>
       <c r="H111" s="2"/>
     </row>
     <row r="112">
       <c r="A112" s="2"/>
-      <c r="B112" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 9</t>
-        </is>
-      </c>
-      <c r="C112" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D112" s="16"/>
-      <c r="E112" s="16"/>
-      <c r="F112" s="16"/>
-      <c r="G112" s="17"/>
+      <c r="B112" s="4"/>
+      <c r="C112" s="5"/>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E112" s="6"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="6"/>
       <c r="H112" s="2"/>
     </row>
     <row r="113">
       <c r="A113" s="2"/>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D113" s="5"/>
+      <c r="B113" s="4"/>
+      <c r="C113" s="5"/>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
-      <c r="G113" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L1 Early Reconstruction; T7 L2 Radical Reconstruction</t>
-        </is>
-      </c>
+      <c r="G113" s="6"/>
       <c r="H113" s="2"/>
     </row>
     <row r="114">
@@ -2408,7 +2464,7 @@
       <c r="C114" s="5"/>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E114" s="6"/>
@@ -2422,7 +2478,7 @@
       <c r="C115" s="5"/>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E115" s="6"/>
@@ -2436,7 +2492,7 @@
       <c r="C116" s="5"/>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E116" s="6"/>
@@ -2446,13 +2502,17 @@
     </row>
     <row r="117">
       <c r="A117" s="2"/>
-      <c r="B117" s="4"/>
-      <c r="C117" s="5"/>
-      <c r="D117" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The War's End</t>
+        </is>
+      </c>
+      <c r="D117" s="5"/>
       <c r="E117" s="6"/>
       <c r="F117" s="6"/>
       <c r="G117" s="6"/>
@@ -2460,84 +2520,80 @@
     </row>
     <row r="118">
       <c r="A118" s="2"/>
-      <c r="B118" s="4"/>
-      <c r="C118" s="5"/>
-      <c r="D118" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E118" s="6"/>
-      <c r="F118" s="6"/>
-      <c r="G118" s="6"/>
+      <c r="B118" s="2"/>
+      <c r="C118" s="2"/>
+      <c r="D118" s="2"/>
+      <c r="E118" s="2"/>
+      <c r="F118" s="2"/>
+      <c r="G118" s="2"/>
       <c r="H118" s="2"/>
     </row>
     <row r="119">
       <c r="A119" s="2"/>
-      <c r="B119" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D119" s="5"/>
-      <c r="E119" s="6"/>
-      <c r="F119" s="6"/>
-      <c r="G119" s="6"/>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 9</t>
+        </is>
+      </c>
+      <c r="C119" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D119" s="16"/>
+      <c r="E119" s="16"/>
+      <c r="F119" s="16"/>
+      <c r="G119" s="17"/>
       <c r="H119" s="2"/>
     </row>
     <row r="120">
       <c r="A120" s="2"/>
-      <c r="B120" s="2"/>
-      <c r="C120" s="2"/>
-      <c r="D120" s="2"/>
-      <c r="E120" s="2"/>
-      <c r="F120" s="2"/>
-      <c r="G120" s="2"/>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D120" s="5"/>
+      <c r="E120" s="6"/>
+      <c r="F120" s="6"/>
+      <c r="G120" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T7 L1 Early Reconstruction; T7 L2 Radical Reconstruction</t>
+        </is>
+      </c>
       <c r="H120" s="2"/>
     </row>
     <row r="121">
       <c r="A121" s="2"/>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 10</t>
-        </is>
-      </c>
-      <c r="C121" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D121" s="16"/>
-      <c r="E121" s="16"/>
-      <c r="F121" s="16"/>
-      <c r="G121" s="17"/>
+      <c r="B121" s="4"/>
+      <c r="C121" s="5"/>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E121" s="6"/>
+      <c r="F121" s="6"/>
+      <c r="G121" s="6"/>
       <c r="H121" s="2"/>
     </row>
     <row r="122">
       <c r="A122" s="2"/>
-      <c r="B122" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C122" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D122" s="5"/>
+      <c r="B122" s="4"/>
+      <c r="C122" s="5"/>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
-      <c r="G122" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L3 Reconstruction and Southern Society; T7 L4 The Aftermath of Reconstruction</t>
-        </is>
-      </c>
+      <c r="G122" s="6"/>
       <c r="H122" s="2"/>
     </row>
     <row r="123">
@@ -2546,7 +2602,7 @@
       <c r="C123" s="5"/>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E123" s="6"/>
@@ -2560,7 +2616,7 @@
       <c r="C124" s="5"/>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E124" s="6"/>
@@ -2574,7 +2630,7 @@
       <c r="C125" s="5"/>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
         </is>
       </c>
       <c r="E125" s="6"/>
@@ -2584,13 +2640,17 @@
     </row>
     <row r="126">
       <c r="A126" s="2"/>
-      <c r="B126" s="4"/>
-      <c r="C126" s="5"/>
-      <c r="D126" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D126" s="5"/>
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
       <c r="G126" s="6"/>
@@ -2598,77 +2658,77 @@
     </row>
     <row r="127">
       <c r="A127" s="2"/>
-      <c r="B127" s="4"/>
-      <c r="C127" s="5"/>
-      <c r="D127" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E127" s="6"/>
-      <c r="F127" s="6"/>
-      <c r="G127" s="6"/>
+      <c r="B127" s="2"/>
+      <c r="C127" s="2"/>
+      <c r="D127" s="2"/>
+      <c r="E127" s="2"/>
+      <c r="F127" s="2"/>
+      <c r="G127" s="2"/>
       <c r="H127" s="2"/>
     </row>
     <row r="128">
       <c r="A128" s="2"/>
-      <c r="B128" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D128" s="5"/>
-      <c r="E128" s="6"/>
-      <c r="F128" s="6"/>
-      <c r="G128" s="6"/>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 10</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D128" s="16"/>
+      <c r="E128" s="16"/>
+      <c r="F128" s="16"/>
+      <c r="G128" s="17"/>
       <c r="H128" s="2"/>
     </row>
     <row r="129">
       <c r="A129" s="2"/>
-      <c r="B129" s="2"/>
-      <c r="C129" s="2"/>
-      <c r="D129" s="2"/>
-      <c r="E129" s="2"/>
-      <c r="F129" s="2"/>
-      <c r="G129" s="2"/>
+      <c r="B129" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D129" s="5"/>
+      <c r="E129" s="6"/>
+      <c r="F129" s="6"/>
+      <c r="G129" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T7 L3 Reconstruction and Southern Society; T7 L4 The Aftermath of Reconstruction</t>
+        </is>
+      </c>
       <c r="H129" s="2"/>
     </row>
     <row r="130">
       <c r="A130" s="2"/>
-      <c r="B130" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 11</t>
-        </is>
-      </c>
-      <c r="C130" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT — Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
-        </is>
-      </c>
-      <c r="D130" s="16"/>
-      <c r="E130" s="16"/>
-      <c r="F130" s="16"/>
-      <c r="G130" s="17"/>
+      <c r="B130" s="4"/>
+      <c r="C130" s="5"/>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E130" s="6"/>
+      <c r="F130" s="6"/>
+      <c r="G130" s="6"/>
       <c r="H130" s="2"/>
     </row>
     <row r="131">
       <c r="A131" s="2"/>
-      <c r="B131" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C131" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
-        </is>
-      </c>
-      <c r="D131" s="5"/>
+      <c r="B131" s="4"/>
+      <c r="C131" s="5"/>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E131" s="6"/>
       <c r="F131" s="6"/>
       <c r="G131" s="6"/>
@@ -2680,7 +2740,7 @@
       <c r="C132" s="5"/>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E132" s="6"/>
@@ -2690,17 +2750,13 @@
     </row>
     <row r="133">
       <c r="A133" s="2"/>
-      <c r="B133" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
-        </is>
-      </c>
-      <c r="D133" s="5"/>
+      <c r="B133" s="4"/>
+      <c r="C133" s="5"/>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
       <c r="G133" s="6"/>
@@ -2708,89 +2764,101 @@
     </row>
     <row r="134">
       <c r="A134" s="2"/>
-      <c r="B134" s="2"/>
-      <c r="C134" s="2"/>
-      <c r="D134" s="2"/>
-      <c r="E134" s="2"/>
-      <c r="F134" s="2"/>
-      <c r="G134" s="2"/>
+      <c r="B134" s="4"/>
+      <c r="C134" s="5"/>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E134" s="6"/>
+      <c r="F134" s="6"/>
+      <c r="G134" s="6"/>
       <c r="H134" s="2"/>
     </row>
     <row r="135">
       <c r="A135" s="2"/>
-      <c r="B135" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 12</t>
-        </is>
-      </c>
-      <c r="C135" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D135" s="16"/>
-      <c r="E135" s="16"/>
-      <c r="F135" s="16"/>
-      <c r="G135" s="17"/>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D135" s="5"/>
+      <c r="E135" s="6"/>
+      <c r="F135" s="6"/>
+      <c r="G135" s="6"/>
       <c r="H135" s="2"/>
     </row>
     <row r="136">
       <c r="A136" s="2"/>
-      <c r="B136" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C136" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D136" s="5"/>
-      <c r="E136" s="6"/>
-      <c r="F136" s="6"/>
-      <c r="G136" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
-        </is>
-      </c>
+      <c r="B136" s="2"/>
+      <c r="C136" s="2"/>
+      <c r="D136" s="2"/>
+      <c r="E136" s="2"/>
+      <c r="F136" s="2"/>
+      <c r="G136" s="2"/>
       <c r="H136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
-      <c r="B137" s="4"/>
-      <c r="C137" s="5"/>
-      <c r="D137" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E137" s="6"/>
-      <c r="F137" s="6"/>
-      <c r="G137" s="6"/>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 11</t>
+        </is>
+      </c>
+      <c r="C137" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
+        </is>
+      </c>
+      <c r="D137" s="16"/>
+      <c r="E137" s="16"/>
+      <c r="F137" s="16"/>
+      <c r="G137" s="17"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138">
       <c r="A138" s="2"/>
-      <c r="B138" s="4"/>
-      <c r="C138" s="5"/>
-      <c r="D138" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT - Was Abraham Lincoln Racist? Academic Debate</t>
+        </is>
+      </c>
+      <c r="D138" s="5"/>
       <c r="E138" s="6"/>
-      <c r="F138" s="6"/>
-      <c r="G138" s="6"/>
+      <c r="F138" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.9.4, 8.9.5, 8.10.4, 8.10.5, 8.11.5 | CCSS-ELA RH.6-8.1, RH.6-8.2, RH.6-8.4, RH.6-8.6, RH.6-8.8, WHST.6-8.1, WHST.6-8.4, WHST.6-8.5, WHST.6-8.6, WHST.6-8.8, WHST.6-8.9, SL.8.4, SL.8.5, SL.8.6 | ELD Part I A.1, Part I A.3, Part I B.5, Part I B.6, Part I B.7, Part I C.10, Part I C.11, Part I C.12</t>
+        </is>
+      </c>
+      <c r="G138" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Was Abraham Lincoln racist?</t>
+        </is>
+      </c>
       <c r="H138" s="2"/>
     </row>
     <row r="139">
       <c r="A139" s="2"/>
-      <c r="B139" s="4"/>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C139" s="5"/>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E139" s="6"/>
@@ -2800,11 +2868,15 @@
     </row>
     <row r="140">
       <c r="A140" s="2"/>
-      <c r="B140" s="4"/>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C140" s="5"/>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E140" s="6"/>
@@ -2814,11 +2886,15 @@
     </row>
     <row r="141">
       <c r="A141" s="2"/>
-      <c r="B141" s="4"/>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C141" s="5"/>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E141" s="6"/>
@@ -2835,7 +2911,7 @@
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
+          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
         </is>
       </c>
       <c r="D142" s="5"/>
@@ -2858,12 +2934,12 @@
       <c r="A144" s="2"/>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 13</t>
+          <t xml:space="preserve">Lesson 12</t>
         </is>
       </c>
       <c r="C144" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hardship for American Indians</t>
+          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D144" s="16"/>
@@ -2881,7 +2957,7 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Hardship for American Indians</t>
+          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D145" s="5"/>
@@ -2889,7 +2965,7 @@
       <c r="F145" s="6"/>
       <c r="G145" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
+          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
         </is>
       </c>
       <c r="H145" s="2"/>
@@ -2973,7 +3049,7 @@
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
+          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D151" s="5"/>
@@ -2996,12 +3072,12 @@
       <c r="A153" s="2"/>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 14</t>
+          <t xml:space="preserve">Lesson 13</t>
         </is>
       </c>
       <c r="C153" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
+          <t xml:space="preserve">Hardship for American Indians</t>
         </is>
       </c>
       <c r="D153" s="16"/>
@@ -3019,7 +3095,7 @@
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
+          <t xml:space="preserve">Overview | Hardship for American Indians</t>
         </is>
       </c>
       <c r="D154" s="5"/>
@@ -3027,7 +3103,7 @@
       <c r="F154" s="6"/>
       <c r="G154" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
+          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
         </is>
       </c>
       <c r="H154" s="2"/>
@@ -3111,7 +3187,7 @@
       </c>
       <c r="C160" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
+          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
         </is>
       </c>
       <c r="D160" s="5"/>
@@ -3134,12 +3210,12 @@
       <c r="A162" s="2"/>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 15</t>
+          <t xml:space="preserve">Lesson 14</t>
         </is>
       </c>
       <c r="C162" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">New Technologies</t>
+          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D162" s="16"/>
@@ -3157,7 +3233,7 @@
       </c>
       <c r="C163" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | New Technologies</t>
+          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D163" s="5"/>
@@ -3165,7 +3241,7 @@
       <c r="F163" s="6"/>
       <c r="G163" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
+          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
         </is>
       </c>
       <c r="H163" s="2"/>
@@ -3249,7 +3325,7 @@
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | New Technologies</t>
+          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D169" s="5"/>
@@ -3272,12 +3348,12 @@
       <c r="A171" s="2"/>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 16</t>
+          <t xml:space="preserve">Lesson 15</t>
         </is>
       </c>
       <c r="C171" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">New Technologies</t>
         </is>
       </c>
       <c r="D171" s="16"/>
@@ -3295,7 +3371,7 @@
       </c>
       <c r="C172" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">Overview | New Technologies</t>
         </is>
       </c>
       <c r="D172" s="5"/>
@@ -3303,7 +3379,7 @@
       <c r="F172" s="6"/>
       <c r="G172" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
+          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
         </is>
       </c>
       <c r="H172" s="2"/>
@@ -3387,7 +3463,7 @@
       </c>
       <c r="C178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">Wrap Up | New Technologies</t>
         </is>
       </c>
       <c r="D178" s="5"/>
@@ -3410,12 +3486,12 @@
       <c r="A180" s="2"/>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 17</t>
+          <t xml:space="preserve">Lesson 16</t>
         </is>
       </c>
       <c r="C180" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Progressive Movement</t>
+          <t xml:space="preserve">Immigration &amp; Urbanization</t>
         </is>
       </c>
       <c r="D180" s="16"/>
@@ -3433,7 +3509,7 @@
       </c>
       <c r="C181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | The Progressive Movement</t>
+          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
         </is>
       </c>
       <c r="D181" s="5"/>
@@ -3441,7 +3517,7 @@
       <c r="F181" s="6"/>
       <c r="G181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
+          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
         </is>
       </c>
       <c r="H181" s="2"/>
@@ -3525,7 +3601,7 @@
       </c>
       <c r="C187" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
+          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
         </is>
       </c>
       <c r="D187" s="5"/>
@@ -3548,12 +3624,12 @@
       <c r="A189" s="2"/>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 18</t>
+          <t xml:space="preserve">Lesson 17</t>
         </is>
       </c>
       <c r="C189" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">The Progressive Movement</t>
         </is>
       </c>
       <c r="D189" s="16"/>
@@ -3571,7 +3647,7 @@
       </c>
       <c r="C190" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Overview | The Progressive Movement</t>
         </is>
       </c>
       <c r="D190" s="5"/>
@@ -3579,7 +3655,7 @@
       <c r="F190" s="6"/>
       <c r="G190" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
+          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
         </is>
       </c>
       <c r="H190" s="2"/>
@@ -3663,7 +3739,7 @@
       </c>
       <c r="C196" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
         </is>
       </c>
       <c r="D196" s="5"/>
@@ -3686,12 +3762,12 @@
       <c r="A198" s="2"/>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 19</t>
+          <t xml:space="preserve">Lesson 18</t>
         </is>
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
         </is>
       </c>
       <c r="D198" s="16"/>
@@ -3709,13 +3785,17 @@
       </c>
       <c r="C199" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
         </is>
       </c>
       <c r="D199" s="5"/>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
-      <c r="G199" s="6"/>
+      <c r="G199" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
+        </is>
+      </c>
       <c r="H199" s="2"/>
     </row>
     <row r="200">
@@ -3724,7 +3804,7 @@
       <c r="C200" s="5"/>
       <c r="D200" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E200" s="6"/>
@@ -3734,17 +3814,13 @@
     </row>
     <row r="201">
       <c r="A201" s="2"/>
-      <c r="B201" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C201" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D201" s="5"/>
+      <c r="B201" s="4"/>
+      <c r="C201" s="5"/>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
       <c r="G201" s="6"/>
@@ -3752,45 +3828,41 @@
     </row>
     <row r="202">
       <c r="A202" s="2"/>
-      <c r="B202" s="2"/>
-      <c r="C202" s="2"/>
-      <c r="D202" s="2"/>
-      <c r="E202" s="2"/>
-      <c r="F202" s="2"/>
-      <c r="G202" s="2"/>
+      <c r="B202" s="4"/>
+      <c r="C202" s="5"/>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E202" s="6"/>
+      <c r="F202" s="6"/>
+      <c r="G202" s="6"/>
       <c r="H202" s="2"/>
     </row>
     <row r="203">
       <c r="A203" s="2"/>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C203" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D203" s="16"/>
-      <c r="E203" s="16"/>
-      <c r="F203" s="16"/>
-      <c r="G203" s="17"/>
+      <c r="B203" s="4"/>
+      <c r="C203" s="5"/>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E203" s="6"/>
+      <c r="F203" s="6"/>
+      <c r="G203" s="6"/>
       <c r="H203" s="2"/>
     </row>
     <row r="204">
       <c r="A204" s="2"/>
-      <c r="B204" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C204" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Final Exam</t>
-        </is>
-      </c>
-      <c r="D204" s="5"/>
+      <c r="B204" s="4"/>
+      <c r="C204" s="5"/>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
       <c r="G204" s="6"/>
@@ -3798,13 +3870,17 @@
     </row>
     <row r="205">
       <c r="A205" s="2"/>
-      <c r="B205" s="4"/>
-      <c r="C205" s="5"/>
-      <c r="D205" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+      <c r="B205" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C205" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D205" s="5"/>
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
       <c r="G205" s="6"/>
@@ -3812,41 +3888,45 @@
     </row>
     <row r="206">
       <c r="A206" s="2"/>
-      <c r="B206" s="4"/>
-      <c r="C206" s="5"/>
-      <c r="D206" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E206" s="6"/>
-      <c r="F206" s="6"/>
-      <c r="G206" s="6"/>
+      <c r="B206" s="2"/>
+      <c r="C206" s="2"/>
+      <c r="D206" s="2"/>
+      <c r="E206" s="2"/>
+      <c r="F206" s="2"/>
+      <c r="G206" s="2"/>
       <c r="H206" s="2"/>
     </row>
     <row r="207">
       <c r="A207" s="2"/>
-      <c r="B207" s="4"/>
-      <c r="C207" s="5"/>
-      <c r="D207" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E207" s="6"/>
-      <c r="F207" s="6"/>
-      <c r="G207" s="6"/>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C207" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D207" s="16"/>
+      <c r="E207" s="16"/>
+      <c r="F207" s="16"/>
+      <c r="G207" s="17"/>
       <c r="H207" s="2"/>
     </row>
     <row r="208">
       <c r="A208" s="2"/>
-      <c r="B208" s="4"/>
-      <c r="C208" s="5"/>
-      <c r="D208" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B208" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C208" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D208" s="5"/>
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
       <c r="G208" s="6"/>
@@ -3858,7 +3938,7 @@
       <c r="C209" s="5"/>
       <c r="D209" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Custom project — detailed outline added when built</t>
         </is>
       </c>
       <c r="E209" s="6"/>
@@ -3875,7 +3955,7 @@
       </c>
       <c r="C210" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Final Exam</t>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
         </is>
       </c>
       <c r="D210" s="5"/>
@@ -3894,6 +3974,140 @@
       <c r="G211" s="2"/>
       <c r="H211" s="2"/>
     </row>
+    <row r="212">
+      <c r="A212" s="2"/>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C212" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D212" s="16"/>
+      <c r="E212" s="16"/>
+      <c r="F212" s="16"/>
+      <c r="G212" s="17"/>
+      <c r="H212" s="2"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="2"/>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C213" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Final Exam</t>
+        </is>
+      </c>
+      <c r="D213" s="5"/>
+      <c r="E213" s="6"/>
+      <c r="F213" s="6"/>
+      <c r="G213" s="6"/>
+      <c r="H213" s="2"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="2"/>
+      <c r="B214" s="4"/>
+      <c r="C214" s="5"/>
+      <c r="D214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E214" s="6"/>
+      <c r="F214" s="6"/>
+      <c r="G214" s="6"/>
+      <c r="H214" s="2"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="2"/>
+      <c r="B215" s="4"/>
+      <c r="C215" s="5"/>
+      <c r="D215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E215" s="6"/>
+      <c r="F215" s="6"/>
+      <c r="G215" s="6"/>
+      <c r="H215" s="2"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="2"/>
+      <c r="B216" s="4"/>
+      <c r="C216" s="5"/>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E216" s="6"/>
+      <c r="F216" s="6"/>
+      <c r="G216" s="6"/>
+      <c r="H216" s="2"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="2"/>
+      <c r="B217" s="4"/>
+      <c r="C217" s="5"/>
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E217" s="6"/>
+      <c r="F217" s="6"/>
+      <c r="G217" s="6"/>
+      <c r="H217" s="2"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="2"/>
+      <c r="B218" s="4"/>
+      <c r="C218" s="5"/>
+      <c r="D218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E218" s="6"/>
+      <c r="F218" s="6"/>
+      <c r="G218" s="6"/>
+      <c r="H218" s="2"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="2"/>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C219" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Final Exam</t>
+        </is>
+      </c>
+      <c r="D219" s="5"/>
+      <c r="E219" s="6"/>
+      <c r="F219" s="6"/>
+      <c r="G219" s="6"/>
+      <c r="H219" s="2"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="2"/>
+      <c r="B220" s="2"/>
+      <c r="C220" s="2"/>
+      <c r="D220" s="2"/>
+      <c r="E220" s="2"/>
+      <c r="F220" s="2"/>
+      <c r="G220" s="2"/>
+      <c r="H220" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="B1:G1"/>
@@ -3903,13 +4117,12 @@
     <mergeCell ref="C45:G45"/>
     <mergeCell ref="C59:G59"/>
     <mergeCell ref="C76:G76"/>
-    <mergeCell ref="C85:G85"/>
-    <mergeCell ref="C94:G94"/>
-    <mergeCell ref="C103:G103"/>
-    <mergeCell ref="C112:G112"/>
-    <mergeCell ref="C121:G121"/>
-    <mergeCell ref="C130:G130"/>
-    <mergeCell ref="C135:G135"/>
+    <mergeCell ref="C92:G92"/>
+    <mergeCell ref="C101:G101"/>
+    <mergeCell ref="C110:G110"/>
+    <mergeCell ref="C119:G119"/>
+    <mergeCell ref="C128:G128"/>
+    <mergeCell ref="C137:G137"/>
     <mergeCell ref="C144:G144"/>
     <mergeCell ref="C153:G153"/>
     <mergeCell ref="C162:G162"/>
@@ -3917,7 +4130,8 @@
     <mergeCell ref="C180:G180"/>
     <mergeCell ref="C189:G189"/>
     <mergeCell ref="C198:G198"/>
-    <mergeCell ref="C203:G203"/>
+    <mergeCell ref="C207:G207"/>
+    <mergeCell ref="C212:G212"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add US History 8-2 Modules 6-10 to dashboard
</commit_message>
<xml_diff>
--- a/exports/US History 8-2 - Course Outline.xlsx
+++ b/exports/US History 8-2 - Course Outline.xlsx
@@ -2146,17 +2146,25 @@
       </c>
       <c r="D93" s="5"/>
       <c r="E93" s="6"/>
-      <c r="F93" s="6"/>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.10.1, 8.10.2, 8.10.3, 8.10.4 | CCSS-ELA RH.1, RH.2, RH.3, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T6 L3 Division and the Outbreak of War; T6 L4 The Course of the War</t>
+          <t xml:space="preserve">Why did the Civil War begin, and how did each side's resources, leaders, strategies, and early battles shape the first years of the war?</t>
         </is>
       </c>
       <c r="H93" s="2"/>
     </row>
     <row r="94">
       <c r="A94" s="2"/>
-      <c r="B94" s="4"/>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C94" s="5"/>
       <c r="D94" s="7" t="inlineStr">
         <is>
@@ -2170,11 +2178,15 @@
     </row>
     <row r="95">
       <c r="A95" s="2"/>
-      <c r="B95" s="4"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C95" s="5"/>
-      <c r="D95" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Division and the Outbreak of War</t>
         </is>
       </c>
       <c r="E95" s="6"/>
@@ -2184,11 +2196,15 @@
     </row>
     <row r="96">
       <c r="A96" s="2"/>
-      <c r="B96" s="4"/>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C96" s="5"/>
-      <c r="D96" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D96" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The Course of the War</t>
         </is>
       </c>
       <c r="E96" s="6"/>
@@ -2198,25 +2214,37 @@
     </row>
     <row r="97">
       <c r="A97" s="2"/>
-      <c r="B97" s="4"/>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C97" s="5"/>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Secession, Fort Sumter, and Early War Strategy</t>
         </is>
       </c>
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
-      <c r="G97" s="6"/>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H97" s="2"/>
     </row>
     <row r="98">
       <c r="A98" s="2"/>
-      <c r="B98" s="4"/>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C98" s="5"/>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E98" s="6"/>
@@ -2228,15 +2256,15 @@
       <c r="A99" s="2"/>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
-        </is>
-      </c>
-      <c r="D99" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C99" s="5"/>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Resources in the North and the South, 1860</t>
+        </is>
+      </c>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
       <c r="G99" s="6"/>
@@ -2244,85 +2272,109 @@
     </row>
     <row r="100">
       <c r="A100" s="2"/>
-      <c r="B100" s="2"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
-      <c r="F100" s="2"/>
-      <c r="G100" s="2"/>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C100" s="5"/>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Abraham Lincoln and Jefferson Davis</t>
+        </is>
+      </c>
+      <c r="E100" s="6"/>
+      <c r="F100" s="6"/>
+      <c r="G100" s="6"/>
       <c r="H100" s="2"/>
     </row>
     <row r="101">
       <c r="A101" s="2"/>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 7</t>
-        </is>
-      </c>
-      <c r="C101" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D101" s="16"/>
-      <c r="E101" s="16"/>
-      <c r="F101" s="16"/>
-      <c r="G101" s="17"/>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C101" s="5"/>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: The Union's Strategies to Win the Civil War</t>
+        </is>
+      </c>
+      <c r="E101" s="6"/>
+      <c r="F101" s="6"/>
+      <c r="G101" s="6"/>
       <c r="H101" s="2"/>
     </row>
     <row r="102">
       <c r="A102" s="2"/>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C102" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D102" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C102" s="5"/>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: Early Battles of the Civil War</t>
+        </is>
+      </c>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
-      <c r="G102" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L5 Emancipation and Life in Wartime</t>
-        </is>
-      </c>
+      <c r="G102" s="6"/>
       <c r="H102" s="2"/>
     </row>
     <row r="103">
       <c r="A103" s="2"/>
-      <c r="B103" s="4"/>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C103" s="5"/>
-      <c r="D103" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
-      <c r="G103" s="6"/>
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H103" s="2"/>
     </row>
     <row r="104">
       <c r="A104" s="2"/>
-      <c r="B104" s="4"/>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C104" s="5"/>
-      <c r="D104" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Battle Where Nobody Died Until the Victory Salute</t>
         </is>
       </c>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="6"/>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H104" s="2"/>
     </row>
     <row r="105">
       <c r="A105" s="2"/>
-      <c r="B105" s="4"/>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C105" s="5"/>
       <c r="D105" s="7" t="inlineStr">
         <is>
@@ -2336,27 +2388,39 @@
     </row>
     <row r="106">
       <c r="A106" s="2"/>
-      <c r="B106" s="4"/>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C106" s="5"/>
-      <c r="D106" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: The Civil War Begins</t>
         </is>
       </c>
       <c r="E106" s="6"/>
       <c r="F106" s="6"/>
-      <c r="G106" s="6"/>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H106" s="2"/>
     </row>
     <row r="107">
       <c r="A107" s="2"/>
-      <c r="B107" s="4"/>
-      <c r="C107" s="5"/>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Civil War Begins</t>
+        </is>
+      </c>
+      <c r="D107" s="5"/>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
       <c r="G107" s="6"/>
@@ -2364,79 +2428,87 @@
     </row>
     <row r="108">
       <c r="A108" s="2"/>
-      <c r="B108" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
-        </is>
-      </c>
-      <c r="D108" s="5"/>
-      <c r="E108" s="6"/>
-      <c r="F108" s="6"/>
-      <c r="G108" s="6"/>
+      <c r="B108" s="2"/>
+      <c r="C108" s="2"/>
+      <c r="D108" s="2"/>
+      <c r="E108" s="2"/>
+      <c r="F108" s="2"/>
+      <c r="G108" s="2"/>
       <c r="H108" s="2"/>
     </row>
     <row r="109">
       <c r="A109" s="2"/>
-      <c r="B109" s="2"/>
-      <c r="C109" s="2"/>
-      <c r="D109" s="2"/>
-      <c r="E109" s="2"/>
-      <c r="F109" s="2"/>
-      <c r="G109" s="2"/>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 7</t>
+        </is>
+      </c>
+      <c r="C109" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D109" s="16"/>
+      <c r="E109" s="16"/>
+      <c r="F109" s="16"/>
+      <c r="G109" s="17"/>
       <c r="H109" s="2"/>
     </row>
     <row r="110">
       <c r="A110" s="2"/>
-      <c r="B110" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 8</t>
-        </is>
-      </c>
-      <c r="C110" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The War's End</t>
-        </is>
-      </c>
-      <c r="D110" s="16"/>
-      <c r="E110" s="16"/>
-      <c r="F110" s="16"/>
-      <c r="G110" s="17"/>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D110" s="5"/>
+      <c r="E110" s="6"/>
+      <c r="F110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.10.4, 8.10.5, 8.11.1 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G110" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did emancipation, African American service, and wartime hardship change the meaning and experience of the Civil War?</t>
+        </is>
+      </c>
       <c r="H110" s="2"/>
     </row>
     <row r="111">
       <c r="A111" s="2"/>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | The War's End</t>
-        </is>
-      </c>
-      <c r="D111" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C111" s="5"/>
+      <c r="D111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E111" s="6"/>
       <c r="F111" s="6"/>
-      <c r="G111" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T6 L6 The War's End</t>
-        </is>
-      </c>
+      <c r="G111" s="6"/>
       <c r="H111" s="2"/>
     </row>
     <row r="112">
       <c r="A112" s="2"/>
-      <c r="B112" s="4"/>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C112" s="5"/>
-      <c r="D112" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Emancipation and Life in Wartime</t>
         </is>
       </c>
       <c r="E112" s="6"/>
@@ -2446,25 +2518,37 @@
     </row>
     <row r="113">
       <c r="A113" s="2"/>
-      <c r="B113" s="4"/>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C113" s="5"/>
-      <c r="D113" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Emancipation and African American Service</t>
         </is>
       </c>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
-      <c r="G113" s="6"/>
+      <c r="G113" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H113" s="2"/>
     </row>
     <row r="114">
       <c r="A114" s="2"/>
-      <c r="B114" s="4"/>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C114" s="5"/>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E114" s="6"/>
@@ -2474,11 +2558,15 @@
     </row>
     <row r="115">
       <c r="A115" s="2"/>
-      <c r="B115" s="4"/>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C115" s="5"/>
-      <c r="D115" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Photography and the Civil War</t>
         </is>
       </c>
       <c r="E115" s="6"/>
@@ -2488,11 +2576,15 @@
     </row>
     <row r="116">
       <c r="A116" s="2"/>
-      <c r="B116" s="4"/>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C116" s="5"/>
-      <c r="D116" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: The Hardships of Soldiers</t>
         </is>
       </c>
       <c r="E116" s="6"/>
@@ -2504,15 +2596,15 @@
       <c r="A117" s="2"/>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The War's End</t>
-        </is>
-      </c>
-      <c r="D117" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C117" s="5"/>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Primary Source: Emancipation Proclamation, Abraham Lincoln</t>
+        </is>
+      </c>
       <c r="E117" s="6"/>
       <c r="F117" s="6"/>
       <c r="G117" s="6"/>
@@ -2520,77 +2612,97 @@
     </row>
     <row r="118">
       <c r="A118" s="2"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="2"/>
-      <c r="D118" s="2"/>
-      <c r="E118" s="2"/>
-      <c r="F118" s="2"/>
-      <c r="G118" s="2"/>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C118" s="5"/>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
+        </is>
+      </c>
+      <c r="E118" s="6"/>
+      <c r="F118" s="6"/>
+      <c r="G118" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H118" s="2"/>
     </row>
     <row r="119">
       <c r="A119" s="2"/>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 9</t>
-        </is>
-      </c>
-      <c r="C119" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D119" s="16"/>
-      <c r="E119" s="16"/>
-      <c r="F119" s="16"/>
-      <c r="G119" s="17"/>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C119" s="5"/>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Enslaved Pilot Who Stole a Confederate Ship</t>
+        </is>
+      </c>
+      <c r="E119" s="6"/>
+      <c r="F119" s="6"/>
+      <c r="G119" s="6"/>
       <c r="H119" s="2"/>
     </row>
     <row r="120">
       <c r="A120" s="2"/>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D120" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C120" s="5"/>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E120" s="6"/>
       <c r="F120" s="6"/>
-      <c r="G120" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L1 Early Reconstruction; T7 L2 Radical Reconstruction</t>
-        </is>
-      </c>
+      <c r="G120" s="6"/>
       <c r="H120" s="2"/>
     </row>
     <row r="121">
       <c r="A121" s="2"/>
-      <c r="B121" s="4"/>
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C121" s="5"/>
-      <c r="D121" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Emancipation &amp; Life in Wartime</t>
         </is>
       </c>
       <c r="E121" s="6"/>
       <c r="F121" s="6"/>
-      <c r="G121" s="6"/>
+      <c r="G121" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H121" s="2"/>
     </row>
     <row r="122">
       <c r="A122" s="2"/>
-      <c r="B122" s="4"/>
-      <c r="C122" s="5"/>
-      <c r="D122" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Emancipation &amp; Life in Wartime</t>
+        </is>
+      </c>
+      <c r="D122" s="5"/>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
       <c r="G122" s="6"/>
@@ -2598,59 +2710,71 @@
     </row>
     <row r="123">
       <c r="A123" s="2"/>
-      <c r="B123" s="4"/>
-      <c r="C123" s="5"/>
-      <c r="D123" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E123" s="6"/>
-      <c r="F123" s="6"/>
-      <c r="G123" s="6"/>
+      <c r="B123" s="2"/>
+      <c r="C123" s="2"/>
+      <c r="D123" s="2"/>
+      <c r="E123" s="2"/>
+      <c r="F123" s="2"/>
+      <c r="G123" s="2"/>
       <c r="H123" s="2"/>
     </row>
     <row r="124">
       <c r="A124" s="2"/>
-      <c r="B124" s="4"/>
-      <c r="C124" s="5"/>
-      <c r="D124" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
-      <c r="E124" s="6"/>
-      <c r="F124" s="6"/>
-      <c r="G124" s="6"/>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 8</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The War's End</t>
+        </is>
+      </c>
+      <c r="D124" s="16"/>
+      <c r="E124" s="16"/>
+      <c r="F124" s="16"/>
+      <c r="G124" s="17"/>
       <c r="H124" s="2"/>
     </row>
     <row r="125">
       <c r="A125" s="2"/>
-      <c r="B125" s="4"/>
-      <c r="C125" s="5"/>
-      <c r="D125" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The War's End</t>
+        </is>
+      </c>
+      <c r="D125" s="5"/>
       <c r="E125" s="6"/>
-      <c r="F125" s="6"/>
-      <c r="G125" s="6"/>
+      <c r="F125" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.10.5, 8.10.6, 8.11.1 | CCSS-ELA RH.1, RH.2, RH.3, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G125" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did major Union victories, total war, and surrender bring the Civil War to an end and force Americans to face the war's cost?</t>
+        </is>
+      </c>
       <c r="H125" s="2"/>
     </row>
     <row r="126">
       <c r="A126" s="2"/>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
-        </is>
-      </c>
-      <c r="D126" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C126" s="5"/>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
       <c r="G126" s="6"/>
@@ -2658,61 +2782,73 @@
     </row>
     <row r="127">
       <c r="A127" s="2"/>
-      <c r="B127" s="2"/>
-      <c r="C127" s="2"/>
-      <c r="D127" s="2"/>
-      <c r="E127" s="2"/>
-      <c r="F127" s="2"/>
-      <c r="G127" s="2"/>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C127" s="5"/>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The War's End</t>
+        </is>
+      </c>
+      <c r="E127" s="6"/>
+      <c r="F127" s="6"/>
+      <c r="G127" s="6"/>
       <c r="H127" s="2"/>
     </row>
     <row r="128">
       <c r="A128" s="2"/>
-      <c r="B128" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 10</t>
-        </is>
-      </c>
-      <c r="C128" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D128" s="16"/>
-      <c r="E128" s="16"/>
-      <c r="F128" s="16"/>
-      <c r="G128" s="17"/>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C128" s="5"/>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Civil War Turning Points and Surrender</t>
+        </is>
+      </c>
+      <c r="E128" s="6"/>
+      <c r="F128" s="6"/>
+      <c r="G128" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H128" s="2"/>
     </row>
     <row r="129">
       <c r="A129" s="2"/>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D129" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C129" s="5"/>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E129" s="6"/>
       <c r="F129" s="6"/>
-      <c r="G129" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T7 L3 Reconstruction and Southern Society; T7 L4 The Aftermath of Reconstruction</t>
-        </is>
-      </c>
+      <c r="G129" s="6"/>
       <c r="H129" s="2"/>
     </row>
     <row r="130">
       <c r="A130" s="2"/>
-      <c r="B130" s="4"/>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C130" s="5"/>
-      <c r="D130" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: The Battle of Vicksburg</t>
         </is>
       </c>
       <c r="E130" s="6"/>
@@ -2722,11 +2858,15 @@
     </row>
     <row r="131">
       <c r="A131" s="2"/>
-      <c r="B131" s="4"/>
+      <c r="B131" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C131" s="5"/>
-      <c r="D131" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3-D Model: The Battle at Gettysburg</t>
         </is>
       </c>
       <c r="E131" s="6"/>
@@ -2736,11 +2876,15 @@
     </row>
     <row r="132">
       <c r="A132" s="2"/>
-      <c r="B132" s="4"/>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C132" s="5"/>
-      <c r="D132" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Key Battles of the Civil War</t>
         </is>
       </c>
       <c r="E132" s="6"/>
@@ -2750,11 +2894,15 @@
     </row>
     <row r="133">
       <c r="A133" s="2"/>
-      <c r="B133" s="4"/>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C133" s="5"/>
-      <c r="D133" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Primary Source: Gettysburg Address, Abraham Lincoln</t>
         </is>
       </c>
       <c r="E133" s="6"/>
@@ -2764,62 +2912,86 @@
     </row>
     <row r="134">
       <c r="A134" s="2"/>
-      <c r="B134" s="4"/>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C134" s="5"/>
-      <c r="D134" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D134" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
-      <c r="G134" s="6"/>
+      <c r="G134" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H134" s="2"/>
     </row>
     <row r="135">
       <c r="A135" s="2"/>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
-        </is>
-      </c>
-      <c r="D135" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C135" s="5"/>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The War That Showed America What Death Looked Like</t>
+        </is>
+      </c>
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
-      <c r="G135" s="6"/>
+      <c r="G135" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H135" s="2"/>
     </row>
     <row r="136">
       <c r="A136" s="2"/>
-      <c r="B136" s="2"/>
-      <c r="C136" s="2"/>
-      <c r="D136" s="2"/>
-      <c r="E136" s="2"/>
-      <c r="F136" s="2"/>
-      <c r="G136" s="2"/>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C136" s="5"/>
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E136" s="6"/>
+      <c r="F136" s="6"/>
+      <c r="G136" s="6"/>
       <c r="H136" s="2"/>
     </row>
     <row r="137">
       <c r="A137" s="2"/>
-      <c r="B137" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 11</t>
-        </is>
-      </c>
-      <c r="C137" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PROJECT - Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
-        </is>
-      </c>
-      <c r="D137" s="16"/>
-      <c r="E137" s="16"/>
-      <c r="F137" s="16"/>
-      <c r="G137" s="17"/>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C137" s="5"/>
+      <c r="D137" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: The War's End</t>
+        </is>
+      </c>
+      <c r="E137" s="6"/>
+      <c r="F137" s="6"/>
+      <c r="G137" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H137" s="2"/>
     </row>
     <row r="138">
@@ -2831,90 +3003,82 @@
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT - Was Abraham Lincoln Racist? Academic Debate</t>
+          <t xml:space="preserve">Wrap Up | The War's End</t>
         </is>
       </c>
       <c r="D138" s="5"/>
       <c r="E138" s="6"/>
-      <c r="F138" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HSS 8.9.4, 8.9.5, 8.10.4, 8.10.5, 8.11.5 | CCSS-ELA RH.6-8.1, RH.6-8.2, RH.6-8.4, RH.6-8.6, RH.6-8.8, WHST.6-8.1, WHST.6-8.4, WHST.6-8.5, WHST.6-8.6, WHST.6-8.8, WHST.6-8.9, SL.8.4, SL.8.5, SL.8.6 | ELD Part I A.1, Part I A.3, Part I B.5, Part I B.6, Part I B.7, Part I C.10, Part I C.11, Part I C.12</t>
-        </is>
-      </c>
-      <c r="G138" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Was Abraham Lincoln racist?</t>
-        </is>
-      </c>
+      <c r="F138" s="6"/>
+      <c r="G138" s="6"/>
       <c r="H138" s="2"/>
     </row>
     <row r="139">
       <c r="A139" s="2"/>
-      <c r="B139" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C139" s="5"/>
-      <c r="D139" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E139" s="6"/>
-      <c r="F139" s="6"/>
-      <c r="G139" s="6"/>
+      <c r="B139" s="2"/>
+      <c r="C139" s="2"/>
+      <c r="D139" s="2"/>
+      <c r="E139" s="2"/>
+      <c r="F139" s="2"/>
+      <c r="G139" s="2"/>
       <c r="H139" s="2"/>
     </row>
     <row r="140">
       <c r="A140" s="2"/>
-      <c r="B140" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C140" s="5"/>
-      <c r="D140" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E140" s="6"/>
-      <c r="F140" s="6"/>
-      <c r="G140" s="6"/>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 9</t>
+        </is>
+      </c>
+      <c r="C140" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D140" s="16"/>
+      <c r="E140" s="16"/>
+      <c r="F140" s="16"/>
+      <c r="G140" s="17"/>
       <c r="H140" s="2"/>
     </row>
     <row r="141">
       <c r="A141" s="2"/>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text Header</t>
-        </is>
-      </c>
-      <c r="C141" s="5"/>
-      <c r="D141" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="D141" s="5"/>
       <c r="E141" s="6"/>
-      <c r="F141" s="6"/>
-      <c r="G141" s="6"/>
+      <c r="F141" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.11.1, 8.11.2, 8.11.3, 8.11.4 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G141" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Reconstruction try to rebuild the nation and redefine freedom, citizenship, and political power after the Civil War?</t>
+        </is>
+      </c>
       <c r="H141" s="2"/>
     </row>
     <row r="142">
       <c r="A142" s="2"/>
       <c r="B142" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
-        </is>
-      </c>
-      <c r="D142" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C142" s="5"/>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E142" s="6"/>
       <c r="F142" s="6"/>
       <c r="G142" s="6"/>
@@ -2922,61 +3086,73 @@
     </row>
     <row r="143">
       <c r="A143" s="2"/>
-      <c r="B143" s="2"/>
-      <c r="C143" s="2"/>
-      <c r="D143" s="2"/>
-      <c r="E143" s="2"/>
-      <c r="F143" s="2"/>
-      <c r="G143" s="2"/>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C143" s="5"/>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Early Reconstruction</t>
+        </is>
+      </c>
+      <c r="E143" s="6"/>
+      <c r="F143" s="6"/>
+      <c r="G143" s="6"/>
       <c r="H143" s="2"/>
     </row>
     <row r="144">
       <c r="A144" s="2"/>
-      <c r="B144" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 12</t>
-        </is>
-      </c>
-      <c r="C144" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D144" s="16"/>
-      <c r="E144" s="16"/>
-      <c r="F144" s="16"/>
-      <c r="G144" s="17"/>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C144" s="5"/>
+      <c r="D144" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="E144" s="6"/>
+      <c r="F144" s="6"/>
+      <c r="G144" s="6"/>
       <c r="H144" s="2"/>
     </row>
     <row r="145">
       <c r="A145" s="2"/>
       <c r="B145" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D145" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C145" s="5"/>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Early and Radical Reconstruction</t>
+        </is>
+      </c>
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
       <c r="G145" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
+          <t xml:space="preserve">6 check questions</t>
         </is>
       </c>
       <c r="H145" s="2"/>
     </row>
     <row r="146">
       <c r="A146" s="2"/>
-      <c r="B146" s="4"/>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C146" s="5"/>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E146" s="6"/>
@@ -2986,11 +3162,15 @@
     </row>
     <row r="147">
       <c r="A147" s="2"/>
-      <c r="B147" s="4"/>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C147" s="5"/>
-      <c r="D147" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Graph: The Downfall of the Southern Economy</t>
         </is>
       </c>
       <c r="E147" s="6"/>
@@ -3000,11 +3180,15 @@
     </row>
     <row r="148">
       <c r="A148" s="2"/>
-      <c r="B148" s="4"/>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C148" s="5"/>
-      <c r="D148" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D148" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Lincoln and Reconstruction</t>
         </is>
       </c>
       <c r="E148" s="6"/>
@@ -3014,11 +3198,15 @@
     </row>
     <row r="149">
       <c r="A149" s="2"/>
-      <c r="B149" s="4"/>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C149" s="5"/>
-      <c r="D149" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D149" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Cartoon: The Massacre of New Orleans</t>
         </is>
       </c>
       <c r="E149" s="6"/>
@@ -3028,62 +3216,86 @@
     </row>
     <row r="150">
       <c r="A150" s="2"/>
-      <c r="B150" s="4"/>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C150" s="5"/>
-      <c r="D150" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D150" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E150" s="6"/>
       <c r="F150" s="6"/>
-      <c r="G150" s="6"/>
+      <c r="G150" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H150" s="2"/>
     </row>
     <row r="151">
       <c r="A151" s="2"/>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D151" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C151" s="5"/>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Formerly Enslaved Man Who Took Jefferson Davis's Senate Seat</t>
+        </is>
+      </c>
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
-      <c r="G151" s="6"/>
+      <c r="G151" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H151" s="2"/>
     </row>
     <row r="152">
       <c r="A152" s="2"/>
-      <c r="B152" s="2"/>
-      <c r="C152" s="2"/>
-      <c r="D152" s="2"/>
-      <c r="E152" s="2"/>
-      <c r="F152" s="2"/>
-      <c r="G152" s="2"/>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C152" s="5"/>
+      <c r="D152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E152" s="6"/>
+      <c r="F152" s="6"/>
+      <c r="G152" s="6"/>
       <c r="H152" s="2"/>
     </row>
     <row r="153">
       <c r="A153" s="2"/>
-      <c r="B153" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 13</t>
-        </is>
-      </c>
-      <c r="C153" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D153" s="16"/>
-      <c r="E153" s="16"/>
-      <c r="F153" s="16"/>
-      <c r="G153" s="17"/>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C153" s="5"/>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Early &amp; Radical Reconstruction</t>
+        </is>
+      </c>
+      <c r="E153" s="6"/>
+      <c r="F153" s="6"/>
+      <c r="G153" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H153" s="2"/>
     </row>
     <row r="154">
@@ -3095,68 +3307,80 @@
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Hardship for American Indians</t>
+          <t xml:space="preserve">Wrap Up | Early &amp; Radical Reconstruction</t>
         </is>
       </c>
       <c r="D154" s="5"/>
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
-      <c r="G154" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
-        </is>
-      </c>
+      <c r="G154" s="6"/>
       <c r="H154" s="2"/>
     </row>
     <row r="155">
       <c r="A155" s="2"/>
-      <c r="B155" s="4"/>
-      <c r="C155" s="5"/>
-      <c r="D155" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E155" s="6"/>
-      <c r="F155" s="6"/>
-      <c r="G155" s="6"/>
+      <c r="B155" s="2"/>
+      <c r="C155" s="2"/>
+      <c r="D155" s="2"/>
+      <c r="E155" s="2"/>
+      <c r="F155" s="2"/>
+      <c r="G155" s="2"/>
       <c r="H155" s="2"/>
     </row>
     <row r="156">
       <c r="A156" s="2"/>
-      <c r="B156" s="4"/>
-      <c r="C156" s="5"/>
-      <c r="D156" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E156" s="6"/>
-      <c r="F156" s="6"/>
-      <c r="G156" s="6"/>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 10</t>
+        </is>
+      </c>
+      <c r="C156" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D156" s="16"/>
+      <c r="E156" s="16"/>
+      <c r="F156" s="16"/>
+      <c r="G156" s="17"/>
       <c r="H156" s="2"/>
     </row>
     <row r="157">
       <c r="A157" s="2"/>
-      <c r="B157" s="4"/>
-      <c r="C157" s="5"/>
-      <c r="D157" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D157" s="5"/>
       <c r="E157" s="6"/>
-      <c r="F157" s="6"/>
-      <c r="G157" s="6"/>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.11.1, 8.11.2, 8.11.3, 8.11.4, 8.11.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.3, Part I B.6.b, Part I B.7</t>
+        </is>
+      </c>
+      <c r="G157" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Reconstruction change southern society, and why did many of its gains collapse or get reversed after federal protection weakened?</t>
+        </is>
+      </c>
       <c r="H157" s="2"/>
     </row>
     <row r="158">
       <c r="A158" s="2"/>
-      <c r="B158" s="4"/>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C158" s="5"/>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E158" s="6"/>
@@ -3166,11 +3390,15 @@
     </row>
     <row r="159">
       <c r="A159" s="2"/>
-      <c r="B159" s="4"/>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C159" s="5"/>
-      <c r="D159" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Reconstruction and Southern Society</t>
         </is>
       </c>
       <c r="E159" s="6"/>
@@ -3182,15 +3410,15 @@
       <c r="A160" s="2"/>
       <c r="B160" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C160" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D160" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C160" s="5"/>
+      <c r="D160" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The Aftermath of Reconstruction</t>
+        </is>
+      </c>
       <c r="E160" s="6"/>
       <c r="F160" s="6"/>
       <c r="G160" s="6"/>
@@ -3198,61 +3426,73 @@
     </row>
     <row r="161">
       <c r="A161" s="2"/>
-      <c r="B161" s="2"/>
-      <c r="C161" s="2"/>
-      <c r="D161" s="2"/>
-      <c r="E161" s="2"/>
-      <c r="F161" s="2"/>
-      <c r="G161" s="2"/>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C161" s="5"/>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Reconstruction Society and the End of Reconstruction</t>
+        </is>
+      </c>
+      <c r="E161" s="6"/>
+      <c r="F161" s="6"/>
+      <c r="G161" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H161" s="2"/>
     </row>
     <row r="162">
       <c r="A162" s="2"/>
-      <c r="B162" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 14</t>
-        </is>
-      </c>
-      <c r="C162" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D162" s="16"/>
-      <c r="E162" s="16"/>
-      <c r="F162" s="16"/>
-      <c r="G162" s="17"/>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C162" s="5"/>
+      <c r="D162" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E162" s="6"/>
+      <c r="F162" s="6"/>
+      <c r="G162" s="6"/>
       <c r="H162" s="2"/>
     </row>
     <row r="163">
       <c r="A163" s="2"/>
       <c r="B163" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C163" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D163" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C163" s="5"/>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Reconstruction-Era Political Groups</t>
+        </is>
+      </c>
       <c r="E163" s="6"/>
       <c r="F163" s="6"/>
-      <c r="G163" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
-        </is>
-      </c>
+      <c r="G163" s="6"/>
       <c r="H163" s="2"/>
     </row>
     <row r="164">
       <c r="A164" s="2"/>
-      <c r="B164" s="4"/>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C164" s="5"/>
-      <c r="D164" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D164" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: The Cycle of Poverty</t>
         </is>
       </c>
       <c r="E164" s="6"/>
@@ -3262,11 +3502,15 @@
     </row>
     <row r="165">
       <c r="A165" s="2"/>
-      <c r="B165" s="4"/>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C165" s="5"/>
-      <c r="D165" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: Oppression of African Americans</t>
         </is>
       </c>
       <c r="E165" s="6"/>
@@ -3276,11 +3520,15 @@
     </row>
     <row r="166">
       <c r="A166" s="2"/>
-      <c r="B166" s="4"/>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C166" s="5"/>
-      <c r="D166" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D166" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Change in Southern Industry</t>
         </is>
       </c>
       <c r="E166" s="6"/>
@@ -3290,45 +3538,61 @@
     </row>
     <row r="167">
       <c r="A167" s="2"/>
-      <c r="B167" s="4"/>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C167" s="5"/>
-      <c r="D167" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
-      <c r="G167" s="6"/>
+      <c r="G167" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 questions</t>
+        </is>
+      </c>
       <c r="H167" s="2"/>
     </row>
     <row r="168">
       <c r="A168" s="2"/>
-      <c r="B168" s="4"/>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C168" s="5"/>
-      <c r="D168" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D168" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The American City Overthrown by a White Supremacist Coup</t>
         </is>
       </c>
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
-      <c r="G168" s="6"/>
+      <c r="G168" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H168" s="2"/>
     </row>
     <row r="169">
       <c r="A169" s="2"/>
       <c r="B169" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C169" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D169" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C169" s="5"/>
+      <c r="D169" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
@@ -3336,89 +3600,109 @@
     </row>
     <row r="170">
       <c r="A170" s="2"/>
-      <c r="B170" s="2"/>
-      <c r="C170" s="2"/>
-      <c r="D170" s="2"/>
-      <c r="E170" s="2"/>
-      <c r="F170" s="2"/>
-      <c r="G170" s="2"/>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C170" s="5"/>
+      <c r="D170" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="E170" s="6"/>
+      <c r="F170" s="6"/>
+      <c r="G170" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H170" s="2"/>
     </row>
     <row r="171">
       <c r="A171" s="2"/>
-      <c r="B171" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 15</t>
-        </is>
-      </c>
-      <c r="C171" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New Technologies</t>
-        </is>
-      </c>
-      <c r="D171" s="16"/>
-      <c r="E171" s="16"/>
-      <c r="F171" s="16"/>
-      <c r="G171" s="17"/>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Reconstruction &amp; Its Aftermath</t>
+        </is>
+      </c>
+      <c r="D171" s="5"/>
+      <c r="E171" s="6"/>
+      <c r="F171" s="6"/>
+      <c r="G171" s="6"/>
       <c r="H171" s="2"/>
     </row>
     <row r="172">
       <c r="A172" s="2"/>
-      <c r="B172" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C172" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | New Technologies</t>
-        </is>
-      </c>
-      <c r="D172" s="5"/>
-      <c r="E172" s="6"/>
-      <c r="F172" s="6"/>
-      <c r="G172" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
-        </is>
-      </c>
+      <c r="B172" s="2"/>
+      <c r="C172" s="2"/>
+      <c r="D172" s="2"/>
+      <c r="E172" s="2"/>
+      <c r="F172" s="2"/>
+      <c r="G172" s="2"/>
       <c r="H172" s="2"/>
     </row>
     <row r="173">
       <c r="A173" s="2"/>
-      <c r="B173" s="4"/>
-      <c r="C173" s="5"/>
-      <c r="D173" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E173" s="6"/>
-      <c r="F173" s="6"/>
-      <c r="G173" s="6"/>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 11</t>
+        </is>
+      </c>
+      <c r="C173" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Was Abraham Lincoln Racist? Academic Debate  (Project)</t>
+        </is>
+      </c>
+      <c r="D173" s="16"/>
+      <c r="E173" s="16"/>
+      <c r="F173" s="16"/>
+      <c r="G173" s="17"/>
       <c r="H173" s="2"/>
     </row>
     <row r="174">
       <c r="A174" s="2"/>
-      <c r="B174" s="4"/>
-      <c r="C174" s="5"/>
-      <c r="D174" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT - Was Abraham Lincoln Racist? Academic Debate</t>
+        </is>
+      </c>
+      <c r="D174" s="5"/>
       <c r="E174" s="6"/>
-      <c r="F174" s="6"/>
-      <c r="G174" s="6"/>
+      <c r="F174" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.9.4, 8.9.5, 8.10.4, 8.10.5, 8.11.5 | CCSS-ELA RH.6-8.1, RH.6-8.2, RH.6-8.4, RH.6-8.6, RH.6-8.8, WHST.6-8.1, WHST.6-8.4, WHST.6-8.5, WHST.6-8.6, WHST.6-8.8, WHST.6-8.9, SL.8.4, SL.8.5, SL.8.6 | ELD Part I A.1, Part I A.3, Part I B.5, Part I B.6, Part I B.7, Part I C.10, Part I C.11, Part I C.12</t>
+        </is>
+      </c>
+      <c r="G174" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Was Abraham Lincoln racist?</t>
+        </is>
+      </c>
       <c r="H174" s="2"/>
     </row>
     <row r="175">
       <c r="A175" s="2"/>
-      <c r="B175" s="4"/>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C175" s="5"/>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E175" s="6"/>
@@ -3428,11 +3712,15 @@
     </row>
     <row r="176">
       <c r="A176" s="2"/>
-      <c r="B176" s="4"/>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C176" s="5"/>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E176" s="6"/>
@@ -3442,11 +3730,15 @@
     </row>
     <row r="177">
       <c r="A177" s="2"/>
-      <c r="B177" s="4"/>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C177" s="5"/>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E177" s="6"/>
@@ -3463,7 +3755,7 @@
       </c>
       <c r="C178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | New Technologies</t>
+          <t xml:space="preserve">Wrap Up | PROJECT — Was Abraham Lincoln Racist? Academic Debate</t>
         </is>
       </c>
       <c r="D178" s="5"/>
@@ -3486,12 +3778,12 @@
       <c r="A180" s="2"/>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 16</t>
+          <t xml:space="preserve">Lesson 12</t>
         </is>
       </c>
       <c r="C180" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D180" s="16"/>
@@ -3509,7 +3801,7 @@
       </c>
       <c r="C181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">Overview | Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D181" s="5"/>
@@ -3517,7 +3809,7 @@
       <c r="F181" s="6"/>
       <c r="G181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
+          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
         </is>
       </c>
       <c r="H181" s="2"/>
@@ -3601,7 +3893,7 @@
       </c>
       <c r="C187" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
+          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="D187" s="5"/>
@@ -3624,12 +3916,12 @@
       <c r="A189" s="2"/>
       <c r="B189" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 17</t>
+          <t xml:space="preserve">Lesson 13</t>
         </is>
       </c>
       <c r="C189" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Progressive Movement</t>
+          <t xml:space="preserve">Hardship for American Indians</t>
         </is>
       </c>
       <c r="D189" s="16"/>
@@ -3647,7 +3939,7 @@
       </c>
       <c r="C190" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | The Progressive Movement</t>
+          <t xml:space="preserve">Overview | Hardship for American Indians</t>
         </is>
       </c>
       <c r="D190" s="5"/>
@@ -3655,7 +3947,7 @@
       <c r="F190" s="6"/>
       <c r="G190" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
+          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
         </is>
       </c>
       <c r="H190" s="2"/>
@@ -3739,7 +4031,7 @@
       </c>
       <c r="C196" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
+          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
         </is>
       </c>
       <c r="D196" s="5"/>
@@ -3762,12 +4054,12 @@
       <c r="A198" s="2"/>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 18</t>
+          <t xml:space="preserve">Lesson 14</t>
         </is>
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D198" s="16"/>
@@ -3785,7 +4077,7 @@
       </c>
       <c r="C199" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D199" s="5"/>
@@ -3793,7 +4085,7 @@
       <c r="F199" s="6"/>
       <c r="G199" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
+          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
         </is>
       </c>
       <c r="H199" s="2"/>
@@ -3877,7 +4169,7 @@
       </c>
       <c r="C205" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D205" s="5"/>
@@ -3900,12 +4192,12 @@
       <c r="A207" s="2"/>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 19</t>
+          <t xml:space="preserve">Lesson 15</t>
         </is>
       </c>
       <c r="C207" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+          <t xml:space="preserve">New Technologies</t>
         </is>
       </c>
       <c r="D207" s="16"/>
@@ -3923,13 +4215,17 @@
       </c>
       <c r="C208" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+          <t xml:space="preserve">Overview | New Technologies</t>
         </is>
       </c>
       <c r="D208" s="5"/>
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
-      <c r="G208" s="6"/>
+      <c r="G208" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
+        </is>
+      </c>
       <c r="H208" s="2"/>
     </row>
     <row r="209">
@@ -3938,7 +4234,7 @@
       <c r="C209" s="5"/>
       <c r="D209" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E209" s="6"/>
@@ -3948,17 +4244,13 @@
     </row>
     <row r="210">
       <c r="A210" s="2"/>
-      <c r="B210" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C210" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D210" s="5"/>
+      <c r="B210" s="4"/>
+      <c r="C210" s="5"/>
+      <c r="D210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E210" s="6"/>
       <c r="F210" s="6"/>
       <c r="G210" s="6"/>
@@ -3966,45 +4258,41 @@
     </row>
     <row r="211">
       <c r="A211" s="2"/>
-      <c r="B211" s="2"/>
-      <c r="C211" s="2"/>
-      <c r="D211" s="2"/>
-      <c r="E211" s="2"/>
-      <c r="F211" s="2"/>
-      <c r="G211" s="2"/>
+      <c r="B211" s="4"/>
+      <c r="C211" s="5"/>
+      <c r="D211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E211" s="6"/>
+      <c r="F211" s="6"/>
+      <c r="G211" s="6"/>
       <c r="H211" s="2"/>
     </row>
     <row r="212">
       <c r="A212" s="2"/>
-      <c r="B212" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C212" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D212" s="16"/>
-      <c r="E212" s="16"/>
-      <c r="F212" s="16"/>
-      <c r="G212" s="17"/>
+      <c r="B212" s="4"/>
+      <c r="C212" s="5"/>
+      <c r="D212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E212" s="6"/>
+      <c r="F212" s="6"/>
+      <c r="G212" s="6"/>
       <c r="H212" s="2"/>
     </row>
     <row r="213">
       <c r="A213" s="2"/>
-      <c r="B213" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C213" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Final Exam</t>
-        </is>
-      </c>
-      <c r="D213" s="5"/>
+      <c r="B213" s="4"/>
+      <c r="C213" s="5"/>
+      <c r="D213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
       <c r="E213" s="6"/>
       <c r="F213" s="6"/>
       <c r="G213" s="6"/>
@@ -4012,13 +4300,17 @@
     </row>
     <row r="214">
       <c r="A214" s="2"/>
-      <c r="B214" s="4"/>
-      <c r="C214" s="5"/>
-      <c r="D214" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C214" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | New Technologies</t>
+        </is>
+      </c>
+      <c r="D214" s="5"/>
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
@@ -4026,44 +4318,52 @@
     </row>
     <row r="215">
       <c r="A215" s="2"/>
-      <c r="B215" s="4"/>
-      <c r="C215" s="5"/>
-      <c r="D215" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E215" s="6"/>
-      <c r="F215" s="6"/>
-      <c r="G215" s="6"/>
+      <c r="B215" s="2"/>
+      <c r="C215" s="2"/>
+      <c r="D215" s="2"/>
+      <c r="E215" s="2"/>
+      <c r="F215" s="2"/>
+      <c r="G215" s="2"/>
       <c r="H215" s="2"/>
     </row>
     <row r="216">
       <c r="A216" s="2"/>
-      <c r="B216" s="4"/>
-      <c r="C216" s="5"/>
-      <c r="D216" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E216" s="6"/>
-      <c r="F216" s="6"/>
-      <c r="G216" s="6"/>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 16</t>
+        </is>
+      </c>
+      <c r="C216" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D216" s="16"/>
+      <c r="E216" s="16"/>
+      <c r="F216" s="16"/>
+      <c r="G216" s="17"/>
       <c r="H216" s="2"/>
     </row>
     <row r="217">
       <c r="A217" s="2"/>
-      <c r="B217" s="4"/>
-      <c r="C217" s="5"/>
-      <c r="D217" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B217" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C217" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D217" s="5"/>
       <c r="E217" s="6"/>
       <c r="F217" s="6"/>
-      <c r="G217" s="6"/>
+      <c r="G217" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
+        </is>
+      </c>
       <c r="H217" s="2"/>
     </row>
     <row r="218">
@@ -4072,7 +4372,7 @@
       <c r="C218" s="5"/>
       <c r="D218" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E218" s="6"/>
@@ -4082,17 +4382,13 @@
     </row>
     <row r="219">
       <c r="A219" s="2"/>
-      <c r="B219" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C219" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Final Exam</t>
-        </is>
-      </c>
-      <c r="D219" s="5"/>
+      <c r="B219" s="4"/>
+      <c r="C219" s="5"/>
+      <c r="D219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E219" s="6"/>
       <c r="F219" s="6"/>
       <c r="G219" s="6"/>
@@ -4100,13 +4396,561 @@
     </row>
     <row r="220">
       <c r="A220" s="2"/>
-      <c r="B220" s="2"/>
-      <c r="C220" s="2"/>
-      <c r="D220" s="2"/>
-      <c r="E220" s="2"/>
-      <c r="F220" s="2"/>
-      <c r="G220" s="2"/>
+      <c r="B220" s="4"/>
+      <c r="C220" s="5"/>
+      <c r="D220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E220" s="6"/>
+      <c r="F220" s="6"/>
+      <c r="G220" s="6"/>
       <c r="H220" s="2"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="2"/>
+      <c r="B221" s="4"/>
+      <c r="C221" s="5"/>
+      <c r="D221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E221" s="6"/>
+      <c r="F221" s="6"/>
+      <c r="G221" s="6"/>
+      <c r="H221" s="2"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2"/>
+      <c r="B222" s="4"/>
+      <c r="C222" s="5"/>
+      <c r="D222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E222" s="6"/>
+      <c r="F222" s="6"/>
+      <c r="G222" s="6"/>
+      <c r="H222" s="2"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2"/>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C223" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D223" s="5"/>
+      <c r="E223" s="6"/>
+      <c r="F223" s="6"/>
+      <c r="G223" s="6"/>
+      <c r="H223" s="2"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2"/>
+      <c r="B224" s="2"/>
+      <c r="C224" s="2"/>
+      <c r="D224" s="2"/>
+      <c r="E224" s="2"/>
+      <c r="F224" s="2"/>
+      <c r="G224" s="2"/>
+      <c r="H224" s="2"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2"/>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 17</t>
+        </is>
+      </c>
+      <c r="C225" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D225" s="16"/>
+      <c r="E225" s="16"/>
+      <c r="F225" s="16"/>
+      <c r="G225" s="17"/>
+      <c r="H225" s="2"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2"/>
+      <c r="B226" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C226" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D226" s="5"/>
+      <c r="E226" s="6"/>
+      <c r="F226" s="6"/>
+      <c r="G226" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
+        </is>
+      </c>
+      <c r="H226" s="2"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2"/>
+      <c r="B227" s="4"/>
+      <c r="C227" s="5"/>
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E227" s="6"/>
+      <c r="F227" s="6"/>
+      <c r="G227" s="6"/>
+      <c r="H227" s="2"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2"/>
+      <c r="B228" s="4"/>
+      <c r="C228" s="5"/>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E228" s="6"/>
+      <c r="F228" s="6"/>
+      <c r="G228" s="6"/>
+      <c r="H228" s="2"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2"/>
+      <c r="B229" s="4"/>
+      <c r="C229" s="5"/>
+      <c r="D229" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E229" s="6"/>
+      <c r="F229" s="6"/>
+      <c r="G229" s="6"/>
+      <c r="H229" s="2"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2"/>
+      <c r="B230" s="4"/>
+      <c r="C230" s="5"/>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E230" s="6"/>
+      <c r="F230" s="6"/>
+      <c r="G230" s="6"/>
+      <c r="H230" s="2"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2"/>
+      <c r="B231" s="4"/>
+      <c r="C231" s="5"/>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E231" s="6"/>
+      <c r="F231" s="6"/>
+      <c r="G231" s="6"/>
+      <c r="H231" s="2"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2"/>
+      <c r="B232" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C232" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D232" s="5"/>
+      <c r="E232" s="6"/>
+      <c r="F232" s="6"/>
+      <c r="G232" s="6"/>
+      <c r="H232" s="2"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2"/>
+      <c r="B233" s="2"/>
+      <c r="C233" s="2"/>
+      <c r="D233" s="2"/>
+      <c r="E233" s="2"/>
+      <c r="F233" s="2"/>
+      <c r="G233" s="2"/>
+      <c r="H233" s="2"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2"/>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 18</t>
+        </is>
+      </c>
+      <c r="C234" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D234" s="16"/>
+      <c r="E234" s="16"/>
+      <c r="F234" s="16"/>
+      <c r="G234" s="17"/>
+      <c r="H234" s="2"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2"/>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C235" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D235" s="5"/>
+      <c r="E235" s="6"/>
+      <c r="F235" s="6"/>
+      <c r="G235" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
+        </is>
+      </c>
+      <c r="H235" s="2"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2"/>
+      <c r="B236" s="4"/>
+      <c r="C236" s="5"/>
+      <c r="D236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E236" s="6"/>
+      <c r="F236" s="6"/>
+      <c r="G236" s="6"/>
+      <c r="H236" s="2"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2"/>
+      <c r="B237" s="4"/>
+      <c r="C237" s="5"/>
+      <c r="D237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E237" s="6"/>
+      <c r="F237" s="6"/>
+      <c r="G237" s="6"/>
+      <c r="H237" s="2"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2"/>
+      <c r="B238" s="4"/>
+      <c r="C238" s="5"/>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E238" s="6"/>
+      <c r="F238" s="6"/>
+      <c r="G238" s="6"/>
+      <c r="H238" s="2"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2"/>
+      <c r="B239" s="4"/>
+      <c r="C239" s="5"/>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E239" s="6"/>
+      <c r="F239" s="6"/>
+      <c r="G239" s="6"/>
+      <c r="H239" s="2"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2"/>
+      <c r="B240" s="4"/>
+      <c r="C240" s="5"/>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E240" s="6"/>
+      <c r="F240" s="6"/>
+      <c r="G240" s="6"/>
+      <c r="H240" s="2"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2"/>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C241" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D241" s="5"/>
+      <c r="E241" s="6"/>
+      <c r="F241" s="6"/>
+      <c r="G241" s="6"/>
+      <c r="H241" s="2"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2"/>
+      <c r="B242" s="2"/>
+      <c r="C242" s="2"/>
+      <c r="D242" s="2"/>
+      <c r="E242" s="2"/>
+      <c r="F242" s="2"/>
+      <c r="G242" s="2"/>
+      <c r="H242" s="2"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2"/>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C243" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D243" s="16"/>
+      <c r="E243" s="16"/>
+      <c r="F243" s="16"/>
+      <c r="G243" s="17"/>
+      <c r="H243" s="2"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2"/>
+      <c r="B244" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C244" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D244" s="5"/>
+      <c r="E244" s="6"/>
+      <c r="F244" s="6"/>
+      <c r="G244" s="6"/>
+      <c r="H244" s="2"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2"/>
+      <c r="B245" s="4"/>
+      <c r="C245" s="5"/>
+      <c r="D245" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+        </is>
+      </c>
+      <c r="E245" s="6"/>
+      <c r="F245" s="6"/>
+      <c r="G245" s="6"/>
+      <c r="H245" s="2"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2"/>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C246" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D246" s="5"/>
+      <c r="E246" s="6"/>
+      <c r="F246" s="6"/>
+      <c r="G246" s="6"/>
+      <c r="H246" s="2"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2"/>
+      <c r="B247" s="2"/>
+      <c r="C247" s="2"/>
+      <c r="D247" s="2"/>
+      <c r="E247" s="2"/>
+      <c r="F247" s="2"/>
+      <c r="G247" s="2"/>
+      <c r="H247" s="2"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2"/>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C248" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D248" s="16"/>
+      <c r="E248" s="16"/>
+      <c r="F248" s="16"/>
+      <c r="G248" s="17"/>
+      <c r="H248" s="2"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2"/>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C249" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Final Exam</t>
+        </is>
+      </c>
+      <c r="D249" s="5"/>
+      <c r="E249" s="6"/>
+      <c r="F249" s="6"/>
+      <c r="G249" s="6"/>
+      <c r="H249" s="2"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2"/>
+      <c r="B250" s="4"/>
+      <c r="C250" s="5"/>
+      <c r="D250" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E250" s="6"/>
+      <c r="F250" s="6"/>
+      <c r="G250" s="6"/>
+      <c r="H250" s="2"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2"/>
+      <c r="B251" s="4"/>
+      <c r="C251" s="5"/>
+      <c r="D251" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E251" s="6"/>
+      <c r="F251" s="6"/>
+      <c r="G251" s="6"/>
+      <c r="H251" s="2"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2"/>
+      <c r="B252" s="4"/>
+      <c r="C252" s="5"/>
+      <c r="D252" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E252" s="6"/>
+      <c r="F252" s="6"/>
+      <c r="G252" s="6"/>
+      <c r="H252" s="2"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2"/>
+      <c r="B253" s="4"/>
+      <c r="C253" s="5"/>
+      <c r="D253" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E253" s="6"/>
+      <c r="F253" s="6"/>
+      <c r="G253" s="6"/>
+      <c r="H253" s="2"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2"/>
+      <c r="B254" s="4"/>
+      <c r="C254" s="5"/>
+      <c r="D254" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[Text Header Title or Topic]</t>
+        </is>
+      </c>
+      <c r="E254" s="6"/>
+      <c r="F254" s="6"/>
+      <c r="G254" s="6"/>
+      <c r="H254" s="2"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2"/>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C255" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Final Exam</t>
+        </is>
+      </c>
+      <c r="D255" s="5"/>
+      <c r="E255" s="6"/>
+      <c r="F255" s="6"/>
+      <c r="G255" s="6"/>
+      <c r="H255" s="2"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2"/>
+      <c r="B256" s="2"/>
+      <c r="C256" s="2"/>
+      <c r="D256" s="2"/>
+      <c r="E256" s="2"/>
+      <c r="F256" s="2"/>
+      <c r="G256" s="2"/>
+      <c r="H256" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -4118,20 +4962,20 @@
     <mergeCell ref="C59:G59"/>
     <mergeCell ref="C76:G76"/>
     <mergeCell ref="C92:G92"/>
-    <mergeCell ref="C101:G101"/>
-    <mergeCell ref="C110:G110"/>
-    <mergeCell ref="C119:G119"/>
-    <mergeCell ref="C128:G128"/>
-    <mergeCell ref="C137:G137"/>
-    <mergeCell ref="C144:G144"/>
-    <mergeCell ref="C153:G153"/>
-    <mergeCell ref="C162:G162"/>
-    <mergeCell ref="C171:G171"/>
+    <mergeCell ref="C109:G109"/>
+    <mergeCell ref="C124:G124"/>
+    <mergeCell ref="C140:G140"/>
+    <mergeCell ref="C156:G156"/>
+    <mergeCell ref="C173:G173"/>
     <mergeCell ref="C180:G180"/>
     <mergeCell ref="C189:G189"/>
     <mergeCell ref="C198:G198"/>
     <mergeCell ref="C207:G207"/>
-    <mergeCell ref="C212:G212"/>
+    <mergeCell ref="C216:G216"/>
+    <mergeCell ref="C225:G225"/>
+    <mergeCell ref="C234:G234"/>
+    <mergeCell ref="C243:G243"/>
+    <mergeCell ref="C248:G248"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update US History 8-2 full reviewer plan
</commit_message>
<xml_diff>
--- a/exports/US History 8-2 - Course Outline.xlsx
+++ b/exports/US History 8-2 - Course Outline.xlsx
@@ -3806,17 +3806,25 @@
       </c>
       <c r="D181" s="5"/>
       <c r="E181" s="6"/>
-      <c r="F181" s="6"/>
+      <c r="F181" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.1, 8.12.2, 8.12.5 | CCSS-ELA RH.1, RH.2, RH.3, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
       <c r="G181" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L1 Mining, Railroads, and the Economy; T8 L2 Western Agriculture</t>
+          <t xml:space="preserve">How did mining, railroads, and farming transform the West, and who paid the highest costs for that expansion?</t>
         </is>
       </c>
       <c r="H181" s="2"/>
     </row>
     <row r="182">
       <c r="A182" s="2"/>
-      <c r="B182" s="4"/>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C182" s="5"/>
       <c r="D182" s="7" t="inlineStr">
         <is>
@@ -3830,11 +3838,15 @@
     </row>
     <row r="183">
       <c r="A183" s="2"/>
-      <c r="B183" s="4"/>
+      <c r="B183" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C183" s="5"/>
-      <c r="D183" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D183" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Mining, Railroads, and the Economy</t>
         </is>
       </c>
       <c r="E183" s="6"/>
@@ -3844,11 +3856,15 @@
     </row>
     <row r="184">
       <c r="A184" s="2"/>
-      <c r="B184" s="4"/>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C184" s="5"/>
-      <c r="D184" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Western Agriculture</t>
         </is>
       </c>
       <c r="E184" s="6"/>
@@ -3858,25 +3874,37 @@
     </row>
     <row r="185">
       <c r="A185" s="2"/>
-      <c r="B185" s="4"/>
+      <c r="B185" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C185" s="5"/>
-      <c r="D185" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D185" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Western Expansion, Railroads, and Homesteading</t>
         </is>
       </c>
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
-      <c r="G185" s="6"/>
+      <c r="G185" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H185" s="2"/>
     </row>
     <row r="186">
       <c r="A186" s="2"/>
-      <c r="B186" s="4"/>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C186" s="5"/>
       <c r="D186" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E186" s="6"/>
@@ -3888,15 +3916,15 @@
       <c r="A187" s="2"/>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C187" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
-        </is>
-      </c>
-      <c r="D187" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C187" s="5"/>
+      <c r="D187" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Boomtowns and Ghost Towns</t>
+        </is>
+      </c>
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
@@ -3904,85 +3932,109 @@
     </row>
     <row r="188">
       <c r="A188" s="2"/>
-      <c r="B188" s="2"/>
-      <c r="C188" s="2"/>
-      <c r="D188" s="2"/>
-      <c r="E188" s="2"/>
-      <c r="F188" s="2"/>
-      <c r="G188" s="2"/>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C188" s="5"/>
+      <c r="D188" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: The Transcontinental Railroad</t>
+        </is>
+      </c>
+      <c r="E188" s="6"/>
+      <c r="F188" s="6"/>
+      <c r="G188" s="6"/>
       <c r="H188" s="2"/>
     </row>
     <row r="189">
       <c r="A189" s="2"/>
-      <c r="B189" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 13</t>
-        </is>
-      </c>
-      <c r="C189" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D189" s="16"/>
-      <c r="E189" s="16"/>
-      <c r="F189" s="16"/>
-      <c r="G189" s="17"/>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C189" s="5"/>
+      <c r="D189" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Cattle Trails</t>
+        </is>
+      </c>
+      <c r="E189" s="6"/>
+      <c r="F189" s="6"/>
+      <c r="G189" s="6"/>
       <c r="H189" s="2"/>
     </row>
     <row r="190">
       <c r="A190" s="2"/>
       <c r="B190" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C190" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D190" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C190" s="5"/>
+      <c r="D190" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3-D Model: Nineteenth-Century Sod House</t>
+        </is>
+      </c>
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
-      <c r="G190" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L3 Hardship for American Indians</t>
-        </is>
-      </c>
+      <c r="G190" s="6"/>
       <c r="H190" s="2"/>
     </row>
     <row r="191">
       <c r="A191" s="2"/>
-      <c r="B191" s="4"/>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C191" s="5"/>
-      <c r="D191" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D191" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
-      <c r="G191" s="6"/>
+      <c r="G191" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
       <c r="H191" s="2"/>
     </row>
     <row r="192">
       <c r="A192" s="2"/>
-      <c r="B192" s="4"/>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C192" s="5"/>
-      <c r="D192" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D192" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Train That Helped Erase the Bison</t>
         </is>
       </c>
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
-      <c r="G192" s="6"/>
+      <c r="G192" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H192" s="2"/>
     </row>
     <row r="193">
       <c r="A193" s="2"/>
-      <c r="B193" s="4"/>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C193" s="5"/>
       <c r="D193" s="7" t="inlineStr">
         <is>
@@ -3996,27 +4048,39 @@
     </row>
     <row r="194">
       <c r="A194" s="2"/>
-      <c r="B194" s="4"/>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C194" s="5"/>
-      <c r="D194" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D194" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Mining, Railroads &amp; Western Agriculture</t>
         </is>
       </c>
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
-      <c r="G194" s="6"/>
+      <c r="G194" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H194" s="2"/>
     </row>
     <row r="195">
       <c r="A195" s="2"/>
-      <c r="B195" s="4"/>
-      <c r="C195" s="5"/>
-      <c r="D195" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B195" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C195" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Mining, Railroads &amp; Western Agriculture</t>
+        </is>
+      </c>
+      <c r="D195" s="5"/>
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
@@ -4024,79 +4088,87 @@
     </row>
     <row r="196">
       <c r="A196" s="2"/>
-      <c r="B196" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C196" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
-        </is>
-      </c>
-      <c r="D196" s="5"/>
-      <c r="E196" s="6"/>
-      <c r="F196" s="6"/>
-      <c r="G196" s="6"/>
+      <c r="B196" s="2"/>
+      <c r="C196" s="2"/>
+      <c r="D196" s="2"/>
+      <c r="E196" s="2"/>
+      <c r="F196" s="2"/>
+      <c r="G196" s="2"/>
       <c r="H196" s="2"/>
     </row>
     <row r="197">
       <c r="A197" s="2"/>
-      <c r="B197" s="2"/>
-      <c r="C197" s="2"/>
-      <c r="D197" s="2"/>
-      <c r="E197" s="2"/>
-      <c r="F197" s="2"/>
-      <c r="G197" s="2"/>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 13</t>
+        </is>
+      </c>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D197" s="16"/>
+      <c r="E197" s="16"/>
+      <c r="F197" s="16"/>
+      <c r="G197" s="17"/>
       <c r="H197" s="2"/>
     </row>
     <row r="198">
       <c r="A198" s="2"/>
-      <c r="B198" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 14</t>
-        </is>
-      </c>
-      <c r="C198" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D198" s="16"/>
-      <c r="E198" s="16"/>
-      <c r="F198" s="16"/>
-      <c r="G198" s="17"/>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C198" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D198" s="5"/>
+      <c r="E198" s="6"/>
+      <c r="F198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.1, 8.12.2, 8.12.3 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G198" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did U.S. expansion and assimilation policies create hardship for American Indian nations and communities?</t>
+        </is>
+      </c>
       <c r="H198" s="2"/>
     </row>
     <row r="199">
       <c r="A199" s="2"/>
       <c r="B199" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C199" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D199" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C199" s="5"/>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
-      <c r="G199" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T8 L4 Industry and Corporations; T8 L5 The Labor Movement</t>
-        </is>
-      </c>
+      <c r="G199" s="6"/>
       <c r="H199" s="2"/>
     </row>
     <row r="200">
       <c r="A200" s="2"/>
-      <c r="B200" s="4"/>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C200" s="5"/>
-      <c r="D200" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Hardship for American Indians</t>
         </is>
       </c>
       <c r="E200" s="6"/>
@@ -4106,25 +4178,37 @@
     </row>
     <row r="201">
       <c r="A201" s="2"/>
-      <c r="B201" s="4"/>
+      <c r="B201" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C201" s="5"/>
-      <c r="D201" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: American Indian Hardship and Assimilation</t>
         </is>
       </c>
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
-      <c r="G201" s="6"/>
+      <c r="G201" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 check questions</t>
+        </is>
+      </c>
       <c r="H201" s="2"/>
     </row>
     <row r="202">
       <c r="A202" s="2"/>
-      <c r="B202" s="4"/>
+      <c r="B202" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C202" s="5"/>
       <c r="D202" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quiz</t>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
         </is>
       </c>
       <c r="E202" s="6"/>
@@ -4134,11 +4218,15 @@
     </row>
     <row r="203">
       <c r="A203" s="2"/>
-      <c r="B203" s="4"/>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C203" s="5"/>
-      <c r="D203" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Native American Losses, 1850-1890</t>
         </is>
       </c>
       <c r="E203" s="6"/>
@@ -4148,11 +4236,15 @@
     </row>
     <row r="204">
       <c r="A204" s="2"/>
-      <c r="B204" s="4"/>
+      <c r="B204" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C204" s="5"/>
-      <c r="D204" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D204" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primary Source: Chief Joseph, I Will Fight No More Forever</t>
         </is>
       </c>
       <c r="E204" s="6"/>
@@ -4164,79 +4256,99 @@
       <c r="A205" s="2"/>
       <c r="B205" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C205" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
-        </is>
-      </c>
-      <c r="D205" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C205" s="5"/>
+      <c r="D205" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
+        </is>
+      </c>
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
-      <c r="G205" s="6"/>
+      <c r="G205" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
       <c r="H205" s="2"/>
     </row>
     <row r="206">
       <c r="A206" s="2"/>
-      <c r="B206" s="2"/>
-      <c r="C206" s="2"/>
-      <c r="D206" s="2"/>
-      <c r="E206" s="2"/>
-      <c r="F206" s="2"/>
-      <c r="G206" s="2"/>
+      <c r="B206" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C206" s="5"/>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: “Kill the Indian, Save the Man”: A Lesson for Children</t>
+        </is>
+      </c>
+      <c r="E206" s="6"/>
+      <c r="F206" s="6"/>
+      <c r="G206" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H206" s="2"/>
     </row>
     <row r="207">
       <c r="A207" s="2"/>
-      <c r="B207" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 15</t>
-        </is>
-      </c>
-      <c r="C207" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">New Technologies</t>
-        </is>
-      </c>
-      <c r="D207" s="16"/>
-      <c r="E207" s="16"/>
-      <c r="F207" s="16"/>
-      <c r="G207" s="17"/>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C207" s="5"/>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E207" s="6"/>
+      <c r="F207" s="6"/>
+      <c r="G207" s="6"/>
       <c r="H207" s="2"/>
     </row>
     <row r="208">
       <c r="A208" s="2"/>
       <c r="B208" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C208" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | New Technologies</t>
-        </is>
-      </c>
-      <c r="D208" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C208" s="5"/>
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Hardship for American Indians</t>
+        </is>
+      </c>
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
       <c r="G208" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Covers: T8 L6 New Technologies</t>
+          <t xml:space="preserve">pool 15, draws 10</t>
         </is>
       </c>
       <c r="H208" s="2"/>
     </row>
     <row r="209">
       <c r="A209" s="2"/>
-      <c r="B209" s="4"/>
-      <c r="C209" s="5"/>
-      <c r="D209" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
+      <c r="B209" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C209" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Hardship for American Indians</t>
+        </is>
+      </c>
+      <c r="D209" s="5"/>
       <c r="E209" s="6"/>
       <c r="F209" s="6"/>
       <c r="G209" s="6"/>
@@ -4244,53 +4356,69 @@
     </row>
     <row r="210">
       <c r="A210" s="2"/>
-      <c r="B210" s="4"/>
-      <c r="C210" s="5"/>
-      <c r="D210" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E210" s="6"/>
-      <c r="F210" s="6"/>
-      <c r="G210" s="6"/>
+      <c r="B210" s="2"/>
+      <c r="C210" s="2"/>
+      <c r="D210" s="2"/>
+      <c r="E210" s="2"/>
+      <c r="F210" s="2"/>
+      <c r="G210" s="2"/>
       <c r="H210" s="2"/>
     </row>
     <row r="211">
       <c r="A211" s="2"/>
-      <c r="B211" s="4"/>
-      <c r="C211" s="5"/>
-      <c r="D211" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
-      <c r="E211" s="6"/>
-      <c r="F211" s="6"/>
-      <c r="G211" s="6"/>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 14</t>
+        </is>
+      </c>
+      <c r="C211" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="D211" s="16"/>
+      <c r="E211" s="16"/>
+      <c r="F211" s="16"/>
+      <c r="G211" s="17"/>
       <c r="H211" s="2"/>
     </row>
     <row r="212">
       <c r="A212" s="2"/>
-      <c r="B212" s="4"/>
-      <c r="C212" s="5"/>
-      <c r="D212" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
-        </is>
-      </c>
+      <c r="B212" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C212" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="D212" s="5"/>
       <c r="E212" s="6"/>
-      <c r="F212" s="6"/>
-      <c r="G212" s="6"/>
+      <c r="F212" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.4, 8.12.5, 8.12.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G212" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did big business change American life, and why did workers organize for better conditions?</t>
+        </is>
+      </c>
       <c r="H212" s="2"/>
     </row>
     <row r="213">
       <c r="A213" s="2"/>
-      <c r="B213" s="4"/>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C213" s="5"/>
       <c r="D213" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E213" s="6"/>
@@ -4302,15 +4430,15 @@
       <c r="A214" s="2"/>
       <c r="B214" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C214" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | New Technologies</t>
-        </is>
-      </c>
-      <c r="D214" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C214" s="5"/>
+      <c r="D214" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Industry and Corporations</t>
+        </is>
+      </c>
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
@@ -4318,61 +4446,73 @@
     </row>
     <row r="215">
       <c r="A215" s="2"/>
-      <c r="B215" s="2"/>
-      <c r="C215" s="2"/>
-      <c r="D215" s="2"/>
-      <c r="E215" s="2"/>
-      <c r="F215" s="2"/>
-      <c r="G215" s="2"/>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C215" s="5"/>
+      <c r="D215" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The Labor Movement</t>
+        </is>
+      </c>
+      <c r="E215" s="6"/>
+      <c r="F215" s="6"/>
+      <c r="G215" s="6"/>
       <c r="H215" s="2"/>
     </row>
     <row r="216">
       <c r="A216" s="2"/>
-      <c r="B216" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 16</t>
-        </is>
-      </c>
-      <c r="C216" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D216" s="16"/>
-      <c r="E216" s="16"/>
-      <c r="F216" s="16"/>
-      <c r="G216" s="17"/>
+      <c r="B216" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C216" s="5"/>
+      <c r="D216" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Big Business and the Labor Movement</t>
+        </is>
+      </c>
+      <c r="E216" s="6"/>
+      <c r="F216" s="6"/>
+      <c r="G216" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
       <c r="H216" s="2"/>
     </row>
     <row r="217">
       <c r="A217" s="2"/>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C217" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D217" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C217" s="5"/>
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E217" s="6"/>
       <c r="F217" s="6"/>
-      <c r="G217" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L1 A New Wave of Immigration; T9 L2 Urbanization</t>
-        </is>
-      </c>
+      <c r="G217" s="6"/>
       <c r="H217" s="2"/>
     </row>
     <row r="218">
       <c r="A218" s="2"/>
-      <c r="B218" s="4"/>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C218" s="5"/>
-      <c r="D218" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D218" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Map: Railroads and Industry</t>
         </is>
       </c>
       <c r="E218" s="6"/>
@@ -4382,11 +4522,15 @@
     </row>
     <row r="219">
       <c r="A219" s="2"/>
-      <c r="B219" s="4"/>
+      <c r="B219" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C219" s="5"/>
-      <c r="D219" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D219" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Advantages and Disadvantages of Big Business</t>
         </is>
       </c>
       <c r="E219" s="6"/>
@@ -4396,11 +4540,15 @@
     </row>
     <row r="220">
       <c r="A220" s="2"/>
-      <c r="B220" s="4"/>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C220" s="5"/>
-      <c r="D220" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D220" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Late 1800s Working Conditions</t>
         </is>
       </c>
       <c r="E220" s="6"/>
@@ -4410,11 +4558,15 @@
     </row>
     <row r="221">
       <c r="A221" s="2"/>
-      <c r="B221" s="4"/>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C221" s="5"/>
-      <c r="D221" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D221" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: The Labor Movement</t>
         </is>
       </c>
       <c r="E221" s="6"/>
@@ -4424,62 +4576,86 @@
     </row>
     <row r="222">
       <c r="A222" s="2"/>
-      <c r="B222" s="4"/>
+      <c r="B222" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C222" s="5"/>
-      <c r="D222" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D222" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E222" s="6"/>
       <c r="F222" s="6"/>
-      <c r="G222" s="6"/>
+      <c r="G222" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
       <c r="H222" s="2"/>
     </row>
     <row r="223">
       <c r="A223" s="2"/>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C223" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
-        </is>
-      </c>
-      <c r="D223" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C223" s="5"/>
+      <c r="D223" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Company That Owned Your Job, Your House, and Your Rent</t>
+        </is>
+      </c>
       <c r="E223" s="6"/>
       <c r="F223" s="6"/>
-      <c r="G223" s="6"/>
+      <c r="G223" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H223" s="2"/>
     </row>
     <row r="224">
       <c r="A224" s="2"/>
-      <c r="B224" s="2"/>
-      <c r="C224" s="2"/>
-      <c r="D224" s="2"/>
-      <c r="E224" s="2"/>
-      <c r="F224" s="2"/>
-      <c r="G224" s="2"/>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C224" s="5"/>
+      <c r="D224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E224" s="6"/>
+      <c r="F224" s="6"/>
+      <c r="G224" s="6"/>
       <c r="H224" s="2"/>
     </row>
     <row r="225">
       <c r="A225" s="2"/>
-      <c r="B225" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 17</t>
-        </is>
-      </c>
-      <c r="C225" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The Progressive Movement</t>
-        </is>
-      </c>
-      <c r="D225" s="16"/>
-      <c r="E225" s="16"/>
-      <c r="F225" s="16"/>
-      <c r="G225" s="17"/>
+      <c r="B225" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C225" s="5"/>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Industry, Corporations &amp; Labor</t>
+        </is>
+      </c>
+      <c r="E225" s="6"/>
+      <c r="F225" s="6"/>
+      <c r="G225" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H225" s="2"/>
     </row>
     <row r="226">
@@ -4491,68 +4667,80 @@
       </c>
       <c r="C226" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | The Progressive Movement</t>
+          <t xml:space="preserve">Wrap Up | Industry, Corporations &amp; Labor</t>
         </is>
       </c>
       <c r="D226" s="5"/>
       <c r="E226" s="6"/>
       <c r="F226" s="6"/>
-      <c r="G226" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L3 The Rise of Progressivism; T9 L4 The Progressive Presidents</t>
-        </is>
-      </c>
+      <c r="G226" s="6"/>
       <c r="H226" s="2"/>
     </row>
     <row r="227">
       <c r="A227" s="2"/>
-      <c r="B227" s="4"/>
-      <c r="C227" s="5"/>
-      <c r="D227" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
-        </is>
-      </c>
-      <c r="E227" s="6"/>
-      <c r="F227" s="6"/>
-      <c r="G227" s="6"/>
+      <c r="B227" s="2"/>
+      <c r="C227" s="2"/>
+      <c r="D227" s="2"/>
+      <c r="E227" s="2"/>
+      <c r="F227" s="2"/>
+      <c r="G227" s="2"/>
       <c r="H227" s="2"/>
     </row>
     <row r="228">
       <c r="A228" s="2"/>
-      <c r="B228" s="4"/>
-      <c r="C228" s="5"/>
-      <c r="D228" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
-        </is>
-      </c>
-      <c r="E228" s="6"/>
-      <c r="F228" s="6"/>
-      <c r="G228" s="6"/>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 15</t>
+        </is>
+      </c>
+      <c r="C228" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New Technologies</t>
+        </is>
+      </c>
+      <c r="D228" s="16"/>
+      <c r="E228" s="16"/>
+      <c r="F228" s="16"/>
+      <c r="G228" s="17"/>
       <c r="H228" s="2"/>
     </row>
     <row r="229">
       <c r="A229" s="2"/>
-      <c r="B229" s="4"/>
-      <c r="C229" s="5"/>
-      <c r="D229" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
-        </is>
-      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | New Technologies</t>
+        </is>
+      </c>
+      <c r="D229" s="5"/>
       <c r="E229" s="6"/>
-      <c r="F229" s="6"/>
-      <c r="G229" s="6"/>
+      <c r="F229" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.5, 8.12.6 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G229" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did new technologies change daily life, business, and Americans’ expectations about the future?</t>
+        </is>
+      </c>
       <c r="H229" s="2"/>
     </row>
     <row r="230">
       <c r="A230" s="2"/>
-      <c r="B230" s="4"/>
+      <c r="B230" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C230" s="5"/>
       <c r="D230" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E230" s="6"/>
@@ -4562,11 +4750,15 @@
     </row>
     <row r="231">
       <c r="A231" s="2"/>
-      <c r="B231" s="4"/>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C231" s="5"/>
-      <c r="D231" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D231" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: New Technologies</t>
         </is>
       </c>
       <c r="E231" s="6"/>
@@ -4578,77 +4770,89 @@
       <c r="A232" s="2"/>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C232" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
-        </is>
-      </c>
-      <c r="D232" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C232" s="5"/>
+      <c r="D232" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Edison, Menlo Park, and New Inventions</t>
+        </is>
+      </c>
       <c r="E232" s="6"/>
       <c r="F232" s="6"/>
-      <c r="G232" s="6"/>
+      <c r="G232" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 check questions</t>
+        </is>
+      </c>
       <c r="H232" s="2"/>
     </row>
     <row r="233">
       <c r="A233" s="2"/>
-      <c r="B233" s="2"/>
-      <c r="C233" s="2"/>
-      <c r="D233" s="2"/>
-      <c r="E233" s="2"/>
-      <c r="F233" s="2"/>
-      <c r="G233" s="2"/>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C233" s="5"/>
+      <c r="D233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E233" s="6"/>
+      <c r="F233" s="6"/>
+      <c r="G233" s="6"/>
       <c r="H233" s="2"/>
     </row>
     <row r="234">
       <c r="A234" s="2"/>
-      <c r="B234" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 18</t>
-        </is>
-      </c>
-      <c r="C234" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
-        </is>
-      </c>
-      <c r="D234" s="16"/>
-      <c r="E234" s="16"/>
-      <c r="F234" s="16"/>
-      <c r="G234" s="17"/>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C234" s="5"/>
+      <c r="D234" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: American Inventors That Changed Society</t>
+        </is>
+      </c>
+      <c r="E234" s="6"/>
+      <c r="F234" s="6"/>
+      <c r="G234" s="6"/>
       <c r="H234" s="2"/>
     </row>
     <row r="235">
       <c r="A235" s="2"/>
       <c r="B235" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C235" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
-        </is>
-      </c>
-      <c r="D235" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C235" s="5"/>
+      <c r="D235" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Inventions Improve Daily Life</t>
+        </is>
+      </c>
       <c r="E235" s="6"/>
       <c r="F235" s="6"/>
-      <c r="G235" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Covers: T9 L5 Progress and Setbacks for Social Justice; T9 L6 A Changing American Culture</t>
-        </is>
-      </c>
+      <c r="G235" s="6"/>
       <c r="H235" s="2"/>
     </row>
     <row r="236">
       <c r="A236" s="2"/>
-      <c r="B236" s="4"/>
+      <c r="B236" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C236" s="5"/>
-      <c r="D236" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D236" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primary Source: Quotations from Thomas Edison</t>
         </is>
       </c>
       <c r="E236" s="6"/>
@@ -4658,39 +4862,59 @@
     </row>
     <row r="237">
       <c r="A237" s="2"/>
-      <c r="B237" s="4"/>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C237" s="5"/>
-      <c r="D237" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D237" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E237" s="6"/>
       <c r="F237" s="6"/>
-      <c r="G237" s="6"/>
+      <c r="G237" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
       <c r="H237" s="2"/>
     </row>
     <row r="238">
       <c r="A238" s="2"/>
-      <c r="B238" s="4"/>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C238" s="5"/>
-      <c r="D238" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D238" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: Can Electricity Cure What Ails You?</t>
         </is>
       </c>
       <c r="E238" s="6"/>
       <c r="F238" s="6"/>
-      <c r="G238" s="6"/>
+      <c r="G238" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H238" s="2"/>
     </row>
     <row r="239">
       <c r="A239" s="2"/>
-      <c r="B239" s="4"/>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C239" s="5"/>
       <c r="D239" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+          <t xml:space="preserve">Quiz</t>
         </is>
       </c>
       <c r="E239" s="6"/>
@@ -4700,16 +4924,24 @@
     </row>
     <row r="240">
       <c r="A240" s="2"/>
-      <c r="B240" s="4"/>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C240" s="5"/>
-      <c r="D240" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D240" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: New Technologies</t>
         </is>
       </c>
       <c r="E240" s="6"/>
       <c r="F240" s="6"/>
-      <c r="G240" s="6"/>
+      <c r="G240" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
       <c r="H240" s="2"/>
     </row>
     <row r="241">
@@ -4721,7 +4953,7 @@
       </c>
       <c r="C241" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+          <t xml:space="preserve">Wrap Up | New Technologies</t>
         </is>
       </c>
       <c r="D241" s="5"/>
@@ -4744,12 +4976,12 @@
       <c r="A243" s="2"/>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lesson 19</t>
+          <t xml:space="preserve">Lesson 16</t>
         </is>
       </c>
       <c r="C243" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROJECT — Current Events Connection  (Project)</t>
+          <t xml:space="preserve">Immigration &amp; Urbanization</t>
         </is>
       </c>
       <c r="D243" s="16"/>
@@ -4767,22 +4999,34 @@
       </c>
       <c r="C244" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Overview | PROJECT — Current Events Connection</t>
+          <t xml:space="preserve">Overview | Immigration &amp; Urbanization</t>
         </is>
       </c>
       <c r="D244" s="5"/>
       <c r="E244" s="6"/>
-      <c r="F244" s="6"/>
-      <c r="G244" s="6"/>
+      <c r="F244" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.6, 8.12.7 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G244" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did immigration and city growth reshape American life in the late 1800s and early 1900s?</t>
+        </is>
+      </c>
       <c r="H244" s="2"/>
     </row>
     <row r="245">
       <c r="A245" s="2"/>
-      <c r="B245" s="4"/>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
       <c r="C245" s="5"/>
       <c r="D245" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Custom project — detailed outline added when built</t>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
         </is>
       </c>
       <c r="E245" s="6"/>
@@ -4794,15 +5038,15 @@
       <c r="A246" s="2"/>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C246" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
-        </is>
-      </c>
-      <c r="D246" s="5"/>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C246" s="5"/>
+      <c r="D246" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: A New Wave of Immigration</t>
+        </is>
+      </c>
       <c r="E246" s="6"/>
       <c r="F246" s="6"/>
       <c r="G246" s="6"/>
@@ -4810,45 +5054,57 @@
     </row>
     <row r="247">
       <c r="A247" s="2"/>
-      <c r="B247" s="2"/>
-      <c r="C247" s="2"/>
-      <c r="D247" s="2"/>
-      <c r="E247" s="2"/>
-      <c r="F247" s="2"/>
-      <c r="G247" s="2"/>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C247" s="5"/>
+      <c r="D247" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Urbanization</t>
+        </is>
+      </c>
+      <c r="E247" s="6"/>
+      <c r="F247" s="6"/>
+      <c r="G247" s="6"/>
       <c r="H247" s="2"/>
     </row>
     <row r="248">
       <c r="A248" s="2"/>
-      <c r="B248" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lesson 20</t>
-        </is>
-      </c>
-      <c r="C248" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Final Exam  (Exam)</t>
-        </is>
-      </c>
-      <c r="D248" s="16"/>
-      <c r="E248" s="16"/>
-      <c r="F248" s="16"/>
-      <c r="G248" s="17"/>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C248" s="5"/>
+      <c r="D248" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Immigration, Cities, and the Gilded Age</t>
+        </is>
+      </c>
+      <c r="E248" s="6"/>
+      <c r="F248" s="6"/>
+      <c r="G248" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 check questions</t>
+        </is>
+      </c>
       <c r="H248" s="2"/>
     </row>
     <row r="249">
       <c r="A249" s="2"/>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C249" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Overview | Final Exam</t>
-        </is>
-      </c>
-      <c r="D249" s="5"/>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C249" s="5"/>
+      <c r="D249" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
       <c r="E249" s="6"/>
       <c r="F249" s="6"/>
       <c r="G249" s="6"/>
@@ -4856,11 +5112,15 @@
     </row>
     <row r="250">
       <c r="A250" s="2"/>
-      <c r="B250" s="4"/>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C250" s="5"/>
-      <c r="D250" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Content and Instructional Assignment</t>
+      <c r="D250" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Immigration, 1870-1910</t>
         </is>
       </c>
       <c r="E250" s="6"/>
@@ -4870,11 +5130,15 @@
     </row>
     <row r="251">
       <c r="A251" s="2"/>
-      <c r="B251" s="4"/>
+      <c r="B251" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C251" s="5"/>
-      <c r="D251" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+      <c r="D251" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Issues Facing Immigrants</t>
         </is>
       </c>
       <c r="E251" s="6"/>
@@ -4884,11 +5148,15 @@
     </row>
     <row r="252">
       <c r="A252" s="2"/>
-      <c r="B252" s="4"/>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C252" s="5"/>
-      <c r="D252" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Quiz</t>
+      <c r="D252" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Urban Problems</t>
         </is>
       </c>
       <c r="E252" s="6"/>
@@ -4898,11 +5166,15 @@
     </row>
     <row r="253">
       <c r="A253" s="2"/>
-      <c r="B253" s="4"/>
+      <c r="B253" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
       <c r="C253" s="5"/>
-      <c r="D253" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D253" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3-D Model: Living in a Tenement</t>
         </is>
       </c>
       <c r="E253" s="6"/>
@@ -4912,45 +5184,1015 @@
     </row>
     <row r="254">
       <c r="A254" s="2"/>
-      <c r="B254" s="4"/>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
       <c r="C254" s="5"/>
-      <c r="D254" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[Text Header Title or Topic]</t>
+      <c r="D254" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
         </is>
       </c>
       <c r="E254" s="6"/>
       <c r="F254" s="6"/>
-      <c r="G254" s="6"/>
+      <c r="G254" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
       <c r="H254" s="2"/>
     </row>
     <row r="255">
       <c r="A255" s="2"/>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page</t>
-        </is>
-      </c>
-      <c r="C255" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wrap Up | Final Exam</t>
-        </is>
-      </c>
-      <c r="D255" s="5"/>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C255" s="5"/>
+      <c r="D255" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The Gang Neighborhood Built on a Poisoned Pond</t>
+        </is>
+      </c>
       <c r="E255" s="6"/>
       <c r="F255" s="6"/>
-      <c r="G255" s="6"/>
+      <c r="G255" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
       <c r="H255" s="2"/>
     </row>
     <row r="256">
       <c r="A256" s="2"/>
-      <c r="B256" s="2"/>
-      <c r="C256" s="2"/>
-      <c r="D256" s="2"/>
-      <c r="E256" s="2"/>
-      <c r="F256" s="2"/>
-      <c r="G256" s="2"/>
+      <c r="B256" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C256" s="5"/>
+      <c r="D256" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E256" s="6"/>
+      <c r="F256" s="6"/>
+      <c r="G256" s="6"/>
       <c r="H256" s="2"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="2"/>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C257" s="5"/>
+      <c r="D257" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="E257" s="6"/>
+      <c r="F257" s="6"/>
+      <c r="G257" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
+      <c r="H257" s="2"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2"/>
+      <c r="B258" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C258" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Immigration &amp; Urbanization</t>
+        </is>
+      </c>
+      <c r="D258" s="5"/>
+      <c r="E258" s="6"/>
+      <c r="F258" s="6"/>
+      <c r="G258" s="6"/>
+      <c r="H258" s="2"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="2"/>
+      <c r="B259" s="2"/>
+      <c r="C259" s="2"/>
+      <c r="D259" s="2"/>
+      <c r="E259" s="2"/>
+      <c r="F259" s="2"/>
+      <c r="G259" s="2"/>
+      <c r="H259" s="2"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="2"/>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 17</t>
+        </is>
+      </c>
+      <c r="C260" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D260" s="16"/>
+      <c r="E260" s="16"/>
+      <c r="F260" s="16"/>
+      <c r="G260" s="17"/>
+      <c r="H260" s="2"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="2"/>
+      <c r="B261" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C261" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D261" s="5"/>
+      <c r="E261" s="6"/>
+      <c r="F261" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.7, 8.12.8, 8.12.9 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G261" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Progressives try to reform government, business, and society?</t>
+        </is>
+      </c>
+      <c r="H261" s="2"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="2"/>
+      <c r="B262" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C262" s="5"/>
+      <c r="D262" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E262" s="6"/>
+      <c r="F262" s="6"/>
+      <c r="G262" s="6"/>
+      <c r="H262" s="2"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2"/>
+      <c r="B263" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C263" s="5"/>
+      <c r="D263" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The Rise of Progressivism</t>
+        </is>
+      </c>
+      <c r="E263" s="6"/>
+      <c r="F263" s="6"/>
+      <c r="G263" s="6"/>
+      <c r="H263" s="2"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2"/>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C264" s="5"/>
+      <c r="D264" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: The Progressive Presidents</t>
+        </is>
+      </c>
+      <c r="E264" s="6"/>
+      <c r="F264" s="6"/>
+      <c r="G264" s="6"/>
+      <c r="H264" s="2"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2"/>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C265" s="5"/>
+      <c r="D265" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Progressive Reform and Progressive Presidents</t>
+        </is>
+      </c>
+      <c r="E265" s="6"/>
+      <c r="F265" s="6"/>
+      <c r="G265" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
+      <c r="H265" s="2"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2"/>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C266" s="5"/>
+      <c r="D266" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E266" s="6"/>
+      <c r="F266" s="6"/>
+      <c r="G266" s="6"/>
+      <c r="H266" s="2"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="2"/>
+      <c r="B267" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C267" s="5"/>
+      <c r="D267" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: Government Reforms in the Progressive Era</t>
+        </is>
+      </c>
+      <c r="E267" s="6"/>
+      <c r="F267" s="6"/>
+      <c r="G267" s="6"/>
+      <c r="H267" s="2"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="2"/>
+      <c r="B268" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C268" s="5"/>
+      <c r="D268" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Progressive Political Reforms</t>
+        </is>
+      </c>
+      <c r="E268" s="6"/>
+      <c r="F268" s="6"/>
+      <c r="G268" s="6"/>
+      <c r="H268" s="2"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2"/>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C269" s="5"/>
+      <c r="D269" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Primary Source: How the Other Half Lives, Jacob Riis</t>
+        </is>
+      </c>
+      <c r="E269" s="6"/>
+      <c r="F269" s="6"/>
+      <c r="G269" s="6"/>
+      <c r="H269" s="2"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="2"/>
+      <c r="B270" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C270" s="5"/>
+      <c r="D270" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Chart: Three Presidents’ Accomplishments</t>
+        </is>
+      </c>
+      <c r="E270" s="6"/>
+      <c r="F270" s="6"/>
+      <c r="G270" s="6"/>
+      <c r="H270" s="2"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2"/>
+      <c r="B271" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C271" s="5"/>
+      <c r="D271" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
+        </is>
+      </c>
+      <c r="E271" s="6"/>
+      <c r="F271" s="6"/>
+      <c r="G271" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
+      <c r="H271" s="2"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="2"/>
+      <c r="B272" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C272" s="5"/>
+      <c r="D272" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: When Food Got So Gross the Government Had to Step In</t>
+        </is>
+      </c>
+      <c r="E272" s="6"/>
+      <c r="F272" s="6"/>
+      <c r="G272" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
+      <c r="H272" s="2"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2"/>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C273" s="5"/>
+      <c r="D273" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E273" s="6"/>
+      <c r="F273" s="6"/>
+      <c r="G273" s="6"/>
+      <c r="H273" s="2"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="2"/>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C274" s="5"/>
+      <c r="D274" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="E274" s="6"/>
+      <c r="F274" s="6"/>
+      <c r="G274" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
+      <c r="H274" s="2"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2"/>
+      <c r="B275" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C275" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | The Progressive Movement</t>
+        </is>
+      </c>
+      <c r="D275" s="5"/>
+      <c r="E275" s="6"/>
+      <c r="F275" s="6"/>
+      <c r="G275" s="6"/>
+      <c r="H275" s="2"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2"/>
+      <c r="B276" s="2"/>
+      <c r="C276" s="2"/>
+      <c r="D276" s="2"/>
+      <c r="E276" s="2"/>
+      <c r="F276" s="2"/>
+      <c r="G276" s="2"/>
+      <c r="H276" s="2"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="2"/>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 18</t>
+        </is>
+      </c>
+      <c r="C277" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D277" s="16"/>
+      <c r="E277" s="16"/>
+      <c r="F277" s="16"/>
+      <c r="G277" s="17"/>
+      <c r="H277" s="2"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2"/>
+      <c r="B278" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C278" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D278" s="5"/>
+      <c r="E278" s="6"/>
+      <c r="F278" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS 8.12.7, 8.12.8, 8.12.9 | CCSS-ELA RH.1, RH.2, RH.3, RH.6, RH.7 | ELD Part I A.1, Part I A.3, Part I B.6</t>
+        </is>
+      </c>
+      <c r="G278" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How did Americans push for social justice and create new cultural forms during the Progressive Era?</t>
+        </is>
+      </c>
+      <c r="H278" s="2"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="2"/>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C279" s="5"/>
+      <c r="D279" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E279" s="6"/>
+      <c r="F279" s="6"/>
+      <c r="G279" s="6"/>
+      <c r="H279" s="2"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2"/>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C280" s="5"/>
+      <c r="D280" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: Progress and Setbacks for Social Justice</t>
+        </is>
+      </c>
+      <c r="E280" s="6"/>
+      <c r="F280" s="6"/>
+      <c r="G280" s="6"/>
+      <c r="H280" s="2"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2"/>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C281" s="5"/>
+      <c r="D281" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eText: A Changing American Culture</t>
+        </is>
+      </c>
+      <c r="E281" s="6"/>
+      <c r="F281" s="6"/>
+      <c r="G281" s="6"/>
+      <c r="H281" s="2"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2"/>
+      <c r="B282" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C282" s="5"/>
+      <c r="D282" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Video: Social Justice and Changing American Culture</t>
+        </is>
+      </c>
+      <c r="E282" s="6"/>
+      <c r="F282" s="6"/>
+      <c r="G282" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 check questions</t>
+        </is>
+      </c>
+      <c r="H282" s="2"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2"/>
+      <c r="B283" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C283" s="5"/>
+      <c r="D283" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E283" s="6"/>
+      <c r="F283" s="6"/>
+      <c r="G283" s="6"/>
+      <c r="H283" s="2"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2"/>
+      <c r="B284" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C284" s="5"/>
+      <c r="D284" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: New Opportunities for Women</t>
+        </is>
+      </c>
+      <c r="E284" s="6"/>
+      <c r="F284" s="6"/>
+      <c r="G284" s="6"/>
+      <c r="H284" s="2"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2"/>
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C285" s="5"/>
+      <c r="D285" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Timeline: African-American Reform Movement, 1895-1915</t>
+        </is>
+      </c>
+      <c r="E285" s="6"/>
+      <c r="F285" s="6"/>
+      <c r="G285" s="6"/>
+      <c r="H285" s="2"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2"/>
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C286" s="5"/>
+      <c r="D286" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: Leisure Activities at the Turn of the Century</t>
+        </is>
+      </c>
+      <c r="E286" s="6"/>
+      <c r="F286" s="6"/>
+      <c r="G286" s="6"/>
+      <c r="H286" s="2"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2"/>
+      <c r="B287" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assignment</t>
+        </is>
+      </c>
+      <c r="C287" s="5"/>
+      <c r="D287" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interactive Gallery: American Realist Artists</t>
+        </is>
+      </c>
+      <c r="E287" s="6"/>
+      <c r="F287" s="6"/>
+      <c r="G287" s="6"/>
+      <c r="H287" s="2"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2"/>
+      <c r="B288" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C288" s="5"/>
+      <c r="D288" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check for Understanding</t>
+        </is>
+      </c>
+      <c r="E288" s="6"/>
+      <c r="F288" s="6"/>
+      <c r="G288" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 questions</t>
+        </is>
+      </c>
+      <c r="H288" s="2"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2"/>
+      <c r="B289" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C289" s="5"/>
+      <c r="D289" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stranger Than Fiction: The President Too Weird to Invent</t>
+        </is>
+      </c>
+      <c r="E289" s="6"/>
+      <c r="F289" s="6"/>
+      <c r="G289" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 questions</t>
+        </is>
+      </c>
+      <c r="H289" s="2"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="2"/>
+      <c r="B290" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C290" s="5"/>
+      <c r="D290" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E290" s="6"/>
+      <c r="F290" s="6"/>
+      <c r="G290" s="6"/>
+      <c r="H290" s="2"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="2"/>
+      <c r="B291" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="C291" s="5"/>
+      <c r="D291" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Module Quiz: Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="E291" s="6"/>
+      <c r="F291" s="6"/>
+      <c r="G291" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool 15, draws 10</t>
+        </is>
+      </c>
+      <c r="H291" s="2"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="2"/>
+      <c r="B292" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C292" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Social Justice &amp; a Changing Culture</t>
+        </is>
+      </c>
+      <c r="D292" s="5"/>
+      <c r="E292" s="6"/>
+      <c r="F292" s="6"/>
+      <c r="G292" s="6"/>
+      <c r="H292" s="2"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="2"/>
+      <c r="B293" s="2"/>
+      <c r="C293" s="2"/>
+      <c r="D293" s="2"/>
+      <c r="E293" s="2"/>
+      <c r="F293" s="2"/>
+      <c r="G293" s="2"/>
+      <c r="H293" s="2"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="2"/>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 19</t>
+        </is>
+      </c>
+      <c r="C294" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROJECT - Current Events Connection  (Project)</t>
+        </is>
+      </c>
+      <c r="D294" s="16"/>
+      <c r="E294" s="16"/>
+      <c r="F294" s="16"/>
+      <c r="G294" s="17"/>
+      <c r="H294" s="2"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="2"/>
+      <c r="B295" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C295" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | PROJECT - Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D295" s="5"/>
+      <c r="E295" s="6"/>
+      <c r="F295" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HSS Course-specific US History 8-2 standards connected to the student-selected current event | CCSS-ELA RH.1, RH.2, RH.6, RH.7, RH.8, W.8.1, W.8.4, W.8.7, W.8.8, W.8.9, SL.8.4, SL.8.5 | ELD Part I A.3, Part I B.6, Part I B.7, Part I C.10, Part I C.11</t>
+        </is>
+      </c>
+      <c r="G295" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How can a current event help us understand patterns, conflicts, and choices from the past?</t>
+        </is>
+      </c>
+      <c r="H295" s="2"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="2"/>
+      <c r="B296" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C296" s="5"/>
+      <c r="D296" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Content and Instructional Assignment</t>
+        </is>
+      </c>
+      <c r="E296" s="6"/>
+      <c r="F296" s="6"/>
+      <c r="G296" s="6"/>
+      <c r="H296" s="2"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="2"/>
+      <c r="B297" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C297" s="5"/>
+      <c r="D297" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reinforcing and Applying Learning</t>
+        </is>
+      </c>
+      <c r="E297" s="6"/>
+      <c r="F297" s="6"/>
+      <c r="G297" s="6"/>
+      <c r="H297" s="2"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="2"/>
+      <c r="B298" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C298" s="5"/>
+      <c r="D298" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quiz</t>
+        </is>
+      </c>
+      <c r="E298" s="6"/>
+      <c r="F298" s="6"/>
+      <c r="G298" s="6"/>
+      <c r="H298" s="2"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="2"/>
+      <c r="B299" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C299" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | PROJECT — Current Events Connection</t>
+        </is>
+      </c>
+      <c r="D299" s="5"/>
+      <c r="E299" s="6"/>
+      <c r="F299" s="6"/>
+      <c r="G299" s="6"/>
+      <c r="H299" s="2"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="2"/>
+      <c r="B300" s="2"/>
+      <c r="C300" s="2"/>
+      <c r="D300" s="2"/>
+      <c r="E300" s="2"/>
+      <c r="F300" s="2"/>
+      <c r="G300" s="2"/>
+      <c r="H300" s="2"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="2"/>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lesson 20</t>
+        </is>
+      </c>
+      <c r="C301" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide &amp; Final Exam  (Exam)</t>
+        </is>
+      </c>
+      <c r="D301" s="16"/>
+      <c r="E301" s="16"/>
+      <c r="F301" s="16"/>
+      <c r="G301" s="17"/>
+      <c r="H301" s="2"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="2"/>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C302" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Overview | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D302" s="5"/>
+      <c r="E302" s="6"/>
+      <c r="F302" s="6"/>
+      <c r="G302" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Semester 2 review and Mastery Connect final exam</t>
+        </is>
+      </c>
+      <c r="H302" s="2"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="2"/>
+      <c r="B303" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C303" s="5"/>
+      <c r="D303" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Study Guide and Final Exam</t>
+        </is>
+      </c>
+      <c r="E303" s="6"/>
+      <c r="F303" s="6"/>
+      <c r="G303" s="6"/>
+      <c r="H303" s="2"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="2"/>
+      <c r="B304" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text Header</t>
+        </is>
+      </c>
+      <c r="C304" s="5"/>
+      <c r="D304" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable / Paper Lesson Guide Source</t>
+        </is>
+      </c>
+      <c r="E304" s="6"/>
+      <c r="F304" s="6"/>
+      <c r="G304" s="6"/>
+      <c r="H304" s="2"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="2"/>
+      <c r="B305" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resource</t>
+        </is>
+      </c>
+      <c r="C305" s="5"/>
+      <c r="D305" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Printable study guide Word document</t>
+        </is>
+      </c>
+      <c r="E305" s="6"/>
+      <c r="F305" s="6"/>
+      <c r="G305" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">US History 8-2 module JSON files 1-19; build tracker; textbook Topic 5 through Topic 9 pages; Mastery Connect final exam when available</t>
+        </is>
+      </c>
+      <c r="H305" s="2"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="2"/>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Page</t>
+        </is>
+      </c>
+      <c r="C306" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wrap Up | Study Guide &amp; Final Exam</t>
+        </is>
+      </c>
+      <c r="D306" s="5"/>
+      <c r="E306" s="6"/>
+      <c r="F306" s="6"/>
+      <c r="G306" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plan now for reviewer website. Build later as a Canvas module with a downloadable study guide and Mastery Connect final exam directions, matching the Semester 1 pattern.</t>
+        </is>
+      </c>
+      <c r="H306" s="2"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="2"/>
+      <c r="B307" s="2"/>
+      <c r="C307" s="2"/>
+      <c r="D307" s="2"/>
+      <c r="E307" s="2"/>
+      <c r="F307" s="2"/>
+      <c r="G307" s="2"/>
+      <c r="H307" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -4968,14 +6210,14 @@
     <mergeCell ref="C156:G156"/>
     <mergeCell ref="C173:G173"/>
     <mergeCell ref="C180:G180"/>
-    <mergeCell ref="C189:G189"/>
-    <mergeCell ref="C198:G198"/>
-    <mergeCell ref="C207:G207"/>
-    <mergeCell ref="C216:G216"/>
-    <mergeCell ref="C225:G225"/>
-    <mergeCell ref="C234:G234"/>
+    <mergeCell ref="C197:G197"/>
+    <mergeCell ref="C211:G211"/>
+    <mergeCell ref="C228:G228"/>
     <mergeCell ref="C243:G243"/>
-    <mergeCell ref="C248:G248"/>
+    <mergeCell ref="C260:G260"/>
+    <mergeCell ref="C277:G277"/>
+    <mergeCell ref="C294:G294"/>
+    <mergeCell ref="C301:G301"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Mastery Connect exam records
</commit_message>
<xml_diff>
--- a/exports/US History 8-2 - Course Outline.xlsx
+++ b/exports/US History 8-2 - Course Outline.xlsx
@@ -6139,7 +6139,7 @@
       <c r="F304" s="6"/>
       <c r="G304" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Your teacher will provide the final exam study guide here after the final exam is confirmed in Mastery Connect. The study guide should be shorter and targeted to the final exam topics.</t>
+          <t xml:space="preserve">Download the study guide, answer the questions in your own words, and study from your answers before the final exam. Download: US History 8-2 Final Exam Study Guide.docx</t>
         </is>
       </c>
       <c r="H304" s="2"/>
@@ -6201,7 +6201,7 @@
       <c r="F307" s="6"/>
       <c r="G307" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Teacher-provided final exam or Mastery Connect blueprint will drive the final study guide later. The old 8-2 PDF guide was reviewed and judged too long for middle school use.</t>
+          <t xml:space="preserve">course_planning/content/8-2/module-20-assets/US-History-8-2-Final-Exam-Study-Guide-CLEAN.docx</t>
         </is>
       </c>
       <c r="H307" s="2"/>
@@ -6223,7 +6223,7 @@
       <c r="F308" s="6"/>
       <c r="G308" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actual Mastery Connect exam is not included here. This module currently contains placeholder directions for the study guide and final exam.</t>
+          <t xml:space="preserve">Mastery Connect Forms A, B, and C are created but remain unavailable and undelivered. This module contains the downloadable study guide and an exam directions placeholder until the team confirms delivery and Canvas tracker setup.</t>
         </is>
       </c>
       <c r="H308" s="2"/>

</xml_diff>